<commit_message>
agg sprint 2 doc
</commit_message>
<xml_diff>
--- a/7_Allegati/Gantt/Gantt_cons.xlsx
+++ b/7_Allegati/Gantt/Gantt_cons.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\M306\Progetto_CasaNote\7_Allegati\Gantt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A655BC61-3FE3-4A66-A51C-C7461E75BC6D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B2CEBFB-B6D0-4FCC-A724-5D0527C84B38}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="14025" xr2:uid="{285B56FD-1A67-4790-99DC-B99A42CD0DBC}"/>
   </bookViews>
@@ -66,9 +66,6 @@
     <t>funzionalità di creazione e gestione del blocco note</t>
   </si>
   <si>
-    <t>Integrazione delle funzionalità di esportazione</t>
-  </si>
-  <si>
     <t xml:space="preserve"> cifratura del database</t>
   </si>
   <si>
@@ -97,6 +94,9 @@
   </si>
   <si>
     <t>Attività</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Integrazione delle funzionalità </t>
   </si>
 </sst>
 </file>
@@ -359,8 +359,23 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -374,35 +389,20 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -726,235 +726,237 @@
   <cols>
     <col min="3" max="3" width="18.85546875" customWidth="1"/>
     <col min="7" max="7" width="22.28515625" customWidth="1"/>
+    <col min="8" max="27" width="9.140625" hidden="1" customWidth="1"/>
+    <col min="28" max="38" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:104" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="24" t="s">
-        <v>23</v>
-      </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24" t="s">
+      <c r="A1" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
-      <c r="K1" s="23"/>
-      <c r="L1" s="23"/>
-      <c r="M1" s="23"/>
-      <c r="N1" s="23"/>
-      <c r="O1" s="23"/>
-      <c r="P1" s="23"/>
-      <c r="Q1" s="23"/>
-      <c r="R1" s="23"/>
-      <c r="S1" s="23"/>
-      <c r="T1" s="23"/>
-      <c r="U1" s="23"/>
-      <c r="V1" s="23"/>
-      <c r="W1" s="23"/>
-      <c r="X1" s="23"/>
-      <c r="Y1" s="23"/>
-      <c r="Z1" s="23"/>
-      <c r="AA1" s="23"/>
-      <c r="AB1" s="23"/>
-      <c r="AC1" s="23"/>
-      <c r="AD1" s="23"/>
-      <c r="AE1" s="23"/>
-      <c r="AF1" s="23"/>
-      <c r="AG1" s="23"/>
-      <c r="AH1" s="23"/>
-      <c r="AI1" s="23"/>
-      <c r="AJ1" s="23"/>
-      <c r="AK1" s="23"/>
-      <c r="AL1" s="23"/>
-      <c r="AM1" s="23"/>
-      <c r="AN1" s="23"/>
-      <c r="AO1" s="23"/>
-      <c r="AP1" s="23"/>
-      <c r="AQ1" s="23"/>
-      <c r="AR1" s="23"/>
-      <c r="AS1" s="23"/>
-      <c r="AT1" s="23"/>
-      <c r="AU1" s="23"/>
-      <c r="AV1" s="23"/>
-      <c r="AW1" s="23"/>
-      <c r="AX1" s="23"/>
-      <c r="AY1" s="23"/>
-      <c r="AZ1" s="23"/>
-      <c r="BA1" s="23"/>
-      <c r="BB1" s="23"/>
-      <c r="BC1" s="23"/>
-      <c r="BD1" s="23"/>
-      <c r="BE1" s="23"/>
-      <c r="BF1" s="23"/>
-      <c r="BG1" s="23"/>
-      <c r="BH1" s="23"/>
-      <c r="BI1" s="23"/>
-      <c r="BJ1" s="23"/>
-      <c r="BK1" s="23"/>
-      <c r="BL1" s="23"/>
-      <c r="BM1" s="23"/>
-      <c r="BN1" s="23"/>
-      <c r="BO1" s="23"/>
-      <c r="BP1" s="23"/>
-      <c r="BQ1" s="23"/>
-      <c r="BR1" s="23"/>
-      <c r="BS1" s="23"/>
-      <c r="BT1" s="23"/>
-      <c r="BU1" s="23"/>
-      <c r="BV1" s="23"/>
-      <c r="BW1" s="23"/>
-      <c r="BX1" s="23"/>
-      <c r="BY1" s="23"/>
-      <c r="BZ1" s="23"/>
-      <c r="CA1" s="23"/>
-      <c r="CB1" s="23"/>
-      <c r="CC1" s="23"/>
-      <c r="CD1" s="23"/>
-      <c r="CE1" s="23"/>
-      <c r="CF1" s="23"/>
-      <c r="CG1" s="23"/>
-      <c r="CH1" s="23"/>
-      <c r="CI1" s="23"/>
-      <c r="CJ1" s="23"/>
-      <c r="CK1" s="23"/>
-      <c r="CL1" s="23"/>
-      <c r="CM1" s="23"/>
-      <c r="CN1" s="23"/>
-      <c r="CO1" s="23"/>
-      <c r="CP1" s="23"/>
-      <c r="CQ1" s="23"/>
-      <c r="CR1" s="23"/>
-      <c r="CS1" s="23"/>
-      <c r="CT1" s="23"/>
-      <c r="CU1" s="23"/>
-      <c r="CV1" s="23"/>
-      <c r="CW1" s="23"/>
-      <c r="CX1" s="23"/>
-      <c r="CY1" s="23"/>
-      <c r="CZ1" s="23"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
+      <c r="J1" s="11"/>
+      <c r="K1" s="11"/>
+      <c r="L1" s="11"/>
+      <c r="M1" s="11"/>
+      <c r="N1" s="11"/>
+      <c r="O1" s="11"/>
+      <c r="P1" s="11"/>
+      <c r="Q1" s="11"/>
+      <c r="R1" s="11"/>
+      <c r="S1" s="11"/>
+      <c r="T1" s="11"/>
+      <c r="U1" s="11"/>
+      <c r="V1" s="11"/>
+      <c r="W1" s="11"/>
+      <c r="X1" s="11"/>
+      <c r="Y1" s="11"/>
+      <c r="Z1" s="11"/>
+      <c r="AA1" s="11"/>
+      <c r="AB1" s="11"/>
+      <c r="AC1" s="11"/>
+      <c r="AD1" s="11"/>
+      <c r="AE1" s="11"/>
+      <c r="AF1" s="11"/>
+      <c r="AG1" s="11"/>
+      <c r="AH1" s="11"/>
+      <c r="AI1" s="11"/>
+      <c r="AJ1" s="11"/>
+      <c r="AK1" s="11"/>
+      <c r="AL1" s="11"/>
+      <c r="AM1" s="11"/>
+      <c r="AN1" s="11"/>
+      <c r="AO1" s="11"/>
+      <c r="AP1" s="11"/>
+      <c r="AQ1" s="11"/>
+      <c r="AR1" s="11"/>
+      <c r="AS1" s="11"/>
+      <c r="AT1" s="11"/>
+      <c r="AU1" s="11"/>
+      <c r="AV1" s="11"/>
+      <c r="AW1" s="11"/>
+      <c r="AX1" s="11"/>
+      <c r="AY1" s="11"/>
+      <c r="AZ1" s="11"/>
+      <c r="BA1" s="11"/>
+      <c r="BB1" s="11"/>
+      <c r="BC1" s="11"/>
+      <c r="BD1" s="11"/>
+      <c r="BE1" s="11"/>
+      <c r="BF1" s="11"/>
+      <c r="BG1" s="11"/>
+      <c r="BH1" s="11"/>
+      <c r="BI1" s="11"/>
+      <c r="BJ1" s="11"/>
+      <c r="BK1" s="11"/>
+      <c r="BL1" s="11"/>
+      <c r="BM1" s="11"/>
+      <c r="BN1" s="11"/>
+      <c r="BO1" s="11"/>
+      <c r="BP1" s="11"/>
+      <c r="BQ1" s="11"/>
+      <c r="BR1" s="11"/>
+      <c r="BS1" s="11"/>
+      <c r="BT1" s="11"/>
+      <c r="BU1" s="11"/>
+      <c r="BV1" s="11"/>
+      <c r="BW1" s="11"/>
+      <c r="BX1" s="11"/>
+      <c r="BY1" s="11"/>
+      <c r="BZ1" s="11"/>
+      <c r="CA1" s="11"/>
+      <c r="CB1" s="11"/>
+      <c r="CC1" s="11"/>
+      <c r="CD1" s="11"/>
+      <c r="CE1" s="11"/>
+      <c r="CF1" s="11"/>
+      <c r="CG1" s="11"/>
+      <c r="CH1" s="11"/>
+      <c r="CI1" s="11"/>
+      <c r="CJ1" s="11"/>
+      <c r="CK1" s="11"/>
+      <c r="CL1" s="11"/>
+      <c r="CM1" s="11"/>
+      <c r="CN1" s="11"/>
+      <c r="CO1" s="11"/>
+      <c r="CP1" s="11"/>
+      <c r="CQ1" s="11"/>
+      <c r="CR1" s="11"/>
+      <c r="CS1" s="11"/>
+      <c r="CT1" s="11"/>
+      <c r="CU1" s="11"/>
+      <c r="CV1" s="11"/>
+      <c r="CW1" s="11"/>
+      <c r="CX1" s="11"/>
+      <c r="CY1" s="11"/>
+      <c r="CZ1" s="11"/>
     </row>
     <row r="2" spans="1:104" ht="16.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="25"/>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
-      <c r="I2" s="23"/>
-      <c r="J2" s="23"/>
-      <c r="K2" s="23"/>
-      <c r="L2" s="23"/>
-      <c r="M2" s="23"/>
-      <c r="N2" s="23"/>
-      <c r="O2" s="23"/>
-      <c r="P2" s="23"/>
-      <c r="Q2" s="23"/>
-      <c r="R2" s="23"/>
-      <c r="S2" s="23"/>
-      <c r="T2" s="23"/>
-      <c r="U2" s="23"/>
-      <c r="V2" s="23"/>
-      <c r="W2" s="23"/>
-      <c r="X2" s="23"/>
-      <c r="Y2" s="23"/>
-      <c r="Z2" s="23"/>
-      <c r="AA2" s="23"/>
-      <c r="AB2" s="23"/>
-      <c r="AC2" s="23"/>
-      <c r="AD2" s="23"/>
-      <c r="AE2" s="23"/>
-      <c r="AF2" s="23"/>
-      <c r="AG2" s="23"/>
-      <c r="AH2" s="23"/>
-      <c r="AI2" s="23"/>
-      <c r="AJ2" s="23"/>
-      <c r="AK2" s="23"/>
-      <c r="AL2" s="23"/>
-      <c r="AM2" s="23"/>
-      <c r="AN2" s="23"/>
-      <c r="AO2" s="23"/>
-      <c r="AP2" s="23"/>
-      <c r="AQ2" s="23"/>
-      <c r="AR2" s="23"/>
-      <c r="AS2" s="23"/>
-      <c r="AT2" s="23"/>
-      <c r="AU2" s="23"/>
-      <c r="AV2" s="23"/>
-      <c r="AW2" s="23"/>
-      <c r="AX2" s="23"/>
-      <c r="AY2" s="23"/>
-      <c r="AZ2" s="23"/>
-      <c r="BA2" s="23"/>
-      <c r="BB2" s="23"/>
-      <c r="BC2" s="23"/>
-      <c r="BD2" s="23"/>
-      <c r="BE2" s="23"/>
-      <c r="BF2" s="23"/>
-      <c r="BG2" s="23"/>
-      <c r="BH2" s="23"/>
-      <c r="BI2" s="23"/>
-      <c r="BJ2" s="23"/>
-      <c r="BK2" s="23"/>
-      <c r="BL2" s="23"/>
-      <c r="BM2" s="23"/>
-      <c r="BN2" s="23"/>
-      <c r="BO2" s="23"/>
-      <c r="BP2" s="23"/>
-      <c r="BQ2" s="23"/>
-      <c r="BR2" s="23"/>
-      <c r="BS2" s="23"/>
-      <c r="BT2" s="23"/>
-      <c r="BU2" s="23"/>
-      <c r="BV2" s="23"/>
-      <c r="BW2" s="23"/>
-      <c r="BX2" s="23"/>
-      <c r="BY2" s="23"/>
-      <c r="BZ2" s="23"/>
-      <c r="CA2" s="23"/>
-      <c r="CB2" s="23"/>
-      <c r="CC2" s="23"/>
-      <c r="CD2" s="23"/>
-      <c r="CE2" s="23"/>
-      <c r="CF2" s="23"/>
-      <c r="CG2" s="23"/>
-      <c r="CH2" s="23"/>
-      <c r="CI2" s="23"/>
-      <c r="CJ2" s="23"/>
-      <c r="CK2" s="23"/>
-      <c r="CL2" s="23"/>
-      <c r="CM2" s="23"/>
-      <c r="CN2" s="23"/>
-      <c r="CO2" s="23"/>
-      <c r="CP2" s="23"/>
-      <c r="CQ2" s="23"/>
-      <c r="CR2" s="23"/>
-      <c r="CS2" s="23"/>
-      <c r="CT2" s="23"/>
-      <c r="CU2" s="23"/>
-      <c r="CV2" s="23"/>
-      <c r="CW2" s="23"/>
-      <c r="CX2" s="23"/>
-      <c r="CY2" s="23"/>
-      <c r="CZ2" s="23"/>
+      <c r="A2" s="13"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="11"/>
+      <c r="H2" s="11"/>
+      <c r="I2" s="11"/>
+      <c r="J2" s="11"/>
+      <c r="K2" s="11"/>
+      <c r="L2" s="11"/>
+      <c r="M2" s="11"/>
+      <c r="N2" s="11"/>
+      <c r="O2" s="11"/>
+      <c r="P2" s="11"/>
+      <c r="Q2" s="11"/>
+      <c r="R2" s="11"/>
+      <c r="S2" s="11"/>
+      <c r="T2" s="11"/>
+      <c r="U2" s="11"/>
+      <c r="V2" s="11"/>
+      <c r="W2" s="11"/>
+      <c r="X2" s="11"/>
+      <c r="Y2" s="11"/>
+      <c r="Z2" s="11"/>
+      <c r="AA2" s="11"/>
+      <c r="AB2" s="11"/>
+      <c r="AC2" s="11"/>
+      <c r="AD2" s="11"/>
+      <c r="AE2" s="11"/>
+      <c r="AF2" s="11"/>
+      <c r="AG2" s="11"/>
+      <c r="AH2" s="11"/>
+      <c r="AI2" s="11"/>
+      <c r="AJ2" s="11"/>
+      <c r="AK2" s="11"/>
+      <c r="AL2" s="11"/>
+      <c r="AM2" s="11"/>
+      <c r="AN2" s="11"/>
+      <c r="AO2" s="11"/>
+      <c r="AP2" s="11"/>
+      <c r="AQ2" s="11"/>
+      <c r="AR2" s="11"/>
+      <c r="AS2" s="11"/>
+      <c r="AT2" s="11"/>
+      <c r="AU2" s="11"/>
+      <c r="AV2" s="11"/>
+      <c r="AW2" s="11"/>
+      <c r="AX2" s="11"/>
+      <c r="AY2" s="11"/>
+      <c r="AZ2" s="11"/>
+      <c r="BA2" s="11"/>
+      <c r="BB2" s="11"/>
+      <c r="BC2" s="11"/>
+      <c r="BD2" s="11"/>
+      <c r="BE2" s="11"/>
+      <c r="BF2" s="11"/>
+      <c r="BG2" s="11"/>
+      <c r="BH2" s="11"/>
+      <c r="BI2" s="11"/>
+      <c r="BJ2" s="11"/>
+      <c r="BK2" s="11"/>
+      <c r="BL2" s="11"/>
+      <c r="BM2" s="11"/>
+      <c r="BN2" s="11"/>
+      <c r="BO2" s="11"/>
+      <c r="BP2" s="11"/>
+      <c r="BQ2" s="11"/>
+      <c r="BR2" s="11"/>
+      <c r="BS2" s="11"/>
+      <c r="BT2" s="11"/>
+      <c r="BU2" s="11"/>
+      <c r="BV2" s="11"/>
+      <c r="BW2" s="11"/>
+      <c r="BX2" s="11"/>
+      <c r="BY2" s="11"/>
+      <c r="BZ2" s="11"/>
+      <c r="CA2" s="11"/>
+      <c r="CB2" s="11"/>
+      <c r="CC2" s="11"/>
+      <c r="CD2" s="11"/>
+      <c r="CE2" s="11"/>
+      <c r="CF2" s="11"/>
+      <c r="CG2" s="11"/>
+      <c r="CH2" s="11"/>
+      <c r="CI2" s="11"/>
+      <c r="CJ2" s="11"/>
+      <c r="CK2" s="11"/>
+      <c r="CL2" s="11"/>
+      <c r="CM2" s="11"/>
+      <c r="CN2" s="11"/>
+      <c r="CO2" s="11"/>
+      <c r="CP2" s="11"/>
+      <c r="CQ2" s="11"/>
+      <c r="CR2" s="11"/>
+      <c r="CS2" s="11"/>
+      <c r="CT2" s="11"/>
+      <c r="CU2" s="11"/>
+      <c r="CV2" s="11"/>
+      <c r="CW2" s="11"/>
+      <c r="CX2" s="11"/>
+      <c r="CY2" s="11"/>
+      <c r="CZ2" s="11"/>
     </row>
     <row r="3" spans="1:104" ht="29.25" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="21">
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="15">
         <v>3</v>
       </c>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="16"/>
       <c r="G3" s="8">
         <v>45665</v>
       </c>
@@ -963,12 +965,12 @@
       <c r="J3" s="1"/>
     </row>
     <row r="4" spans="1:104" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A4" s="20"/>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
+      <c r="A4" s="14"/>
+      <c r="B4" s="14"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="16"/>
       <c r="G4" s="9">
         <v>45665</v>
       </c>
@@ -977,16 +979,16 @@
       <c r="J4" s="1"/>
     </row>
     <row r="5" spans="1:104" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="20" t="s">
+      <c r="A5" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="20"/>
-      <c r="C5" s="20"/>
-      <c r="D5" s="21">
+      <c r="B5" s="14"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="15">
         <v>3</v>
       </c>
-      <c r="E5" s="22"/>
-      <c r="F5" s="22"/>
+      <c r="E5" s="16"/>
+      <c r="F5" s="16"/>
       <c r="G5" s="9">
         <v>45665</v>
       </c>
@@ -995,12 +997,12 @@
       <c r="M5" s="1"/>
     </row>
     <row r="6" spans="1:104" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A6" s="20"/>
-      <c r="B6" s="20"/>
-      <c r="C6" s="20"/>
-      <c r="D6" s="21"/>
-      <c r="E6" s="22"/>
-      <c r="F6" s="22"/>
+      <c r="A6" s="14"/>
+      <c r="B6" s="14"/>
+      <c r="C6" s="14"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="16"/>
       <c r="G6" s="9">
         <v>45665</v>
       </c>
@@ -1009,16 +1011,16 @@
       <c r="M6" s="1"/>
     </row>
     <row r="7" spans="1:104" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A7" s="20" t="s">
+      <c r="A7" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="20"/>
-      <c r="C7" s="20"/>
-      <c r="D7" s="12">
+      <c r="B7" s="14"/>
+      <c r="C7" s="14"/>
+      <c r="D7" s="17">
         <v>3</v>
       </c>
-      <c r="E7" s="12"/>
-      <c r="F7" s="13"/>
+      <c r="E7" s="17"/>
+      <c r="F7" s="18"/>
       <c r="G7" s="10">
         <v>45665</v>
       </c>
@@ -1027,12 +1029,12 @@
       <c r="P7" s="1"/>
     </row>
     <row r="8" spans="1:104" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A8" s="20"/>
-      <c r="B8" s="20"/>
-      <c r="C8" s="20"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="15"/>
+      <c r="A8" s="14"/>
+      <c r="B8" s="14"/>
+      <c r="C8" s="14"/>
+      <c r="D8" s="19"/>
+      <c r="E8" s="19"/>
+      <c r="F8" s="20"/>
       <c r="G8" s="10">
         <v>45672</v>
       </c>
@@ -1041,16 +1043,16 @@
       <c r="P8" s="1"/>
     </row>
     <row r="9" spans="1:104" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="19"/>
-      <c r="C9" s="19"/>
-      <c r="D9" s="12">
+      <c r="B9" s="21"/>
+      <c r="C9" s="21"/>
+      <c r="D9" s="17">
         <v>2</v>
       </c>
-      <c r="E9" s="12"/>
-      <c r="F9" s="13"/>
+      <c r="E9" s="17"/>
+      <c r="F9" s="18"/>
       <c r="G9" s="9">
         <v>45672</v>
       </c>
@@ -1059,12 +1061,12 @@
       <c r="S9" s="2"/>
     </row>
     <row r="10" spans="1:104" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A10" s="19"/>
-      <c r="B10" s="19"/>
-      <c r="C10" s="19"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="14"/>
-      <c r="F10" s="15"/>
+      <c r="A10" s="21"/>
+      <c r="B10" s="21"/>
+      <c r="C10" s="21"/>
+      <c r="D10" s="19"/>
+      <c r="E10" s="19"/>
+      <c r="F10" s="20"/>
       <c r="G10" s="9">
         <v>45679</v>
       </c>
@@ -1073,16 +1075,16 @@
       <c r="S10" s="2"/>
     </row>
     <row r="11" spans="1:104" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="B11" s="19"/>
-      <c r="C11" s="19"/>
-      <c r="D11" s="12">
+      <c r="B11" s="21"/>
+      <c r="C11" s="21"/>
+      <c r="D11" s="17">
         <v>2</v>
       </c>
-      <c r="E11" s="12"/>
-      <c r="F11" s="13"/>
+      <c r="E11" s="17"/>
+      <c r="F11" s="18"/>
       <c r="G11" s="9">
         <v>45672</v>
       </c>
@@ -1090,12 +1092,12 @@
       <c r="U11" s="2"/>
     </row>
     <row r="12" spans="1:104" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A12" s="19"/>
-      <c r="B12" s="19"/>
-      <c r="C12" s="19"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="15"/>
+      <c r="A12" s="21"/>
+      <c r="B12" s="21"/>
+      <c r="C12" s="21"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="20"/>
       <c r="G12" s="9">
         <v>45679</v>
       </c>
@@ -1103,16 +1105,16 @@
       <c r="U12" s="2"/>
     </row>
     <row r="13" spans="1:104" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A13" s="19" t="s">
+      <c r="A13" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="B13" s="19"/>
-      <c r="C13" s="19"/>
-      <c r="D13" s="12">
+      <c r="B13" s="21"/>
+      <c r="C13" s="21"/>
+      <c r="D13" s="17">
         <v>2</v>
       </c>
-      <c r="E13" s="12"/>
-      <c r="F13" s="13"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="18"/>
       <c r="G13" s="9">
         <v>45672</v>
       </c>
@@ -1120,12 +1122,12 @@
       <c r="W13" s="2"/>
     </row>
     <row r="14" spans="1:104" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A14" s="19"/>
-      <c r="B14" s="19"/>
-      <c r="C14" s="19"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="15"/>
+      <c r="A14" s="21"/>
+      <c r="B14" s="21"/>
+      <c r="C14" s="21"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="20"/>
       <c r="G14" s="9">
         <v>45679</v>
       </c>
@@ -1133,16 +1135,16 @@
       <c r="W14" s="2"/>
     </row>
     <row r="15" spans="1:104" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A15" s="19" t="s">
+      <c r="A15" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="B15" s="19"/>
-      <c r="C15" s="19"/>
-      <c r="D15" s="12">
+      <c r="B15" s="21"/>
+      <c r="C15" s="21"/>
+      <c r="D15" s="17">
         <v>2</v>
       </c>
-      <c r="E15" s="12"/>
-      <c r="F15" s="13"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="18"/>
       <c r="G15" s="9">
         <v>45679</v>
       </c>
@@ -1150,12 +1152,12 @@
       <c r="Y15" s="2"/>
     </row>
     <row r="16" spans="1:104" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A16" s="19"/>
-      <c r="B16" s="19"/>
-      <c r="C16" s="19"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14"/>
-      <c r="F16" s="15"/>
+      <c r="A16" s="21"/>
+      <c r="B16" s="21"/>
+      <c r="C16" s="21"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="20"/>
       <c r="G16" s="10">
         <v>45693</v>
       </c>
@@ -1163,16 +1165,16 @@
       <c r="Y16" s="2"/>
     </row>
     <row r="17" spans="1:62" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A17" s="19" t="s">
+      <c r="A17" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="B17" s="19"/>
-      <c r="C17" s="19"/>
-      <c r="D17" s="12">
+      <c r="B17" s="21"/>
+      <c r="C17" s="21"/>
+      <c r="D17" s="17">
         <v>2</v>
       </c>
-      <c r="E17" s="12"/>
-      <c r="F17" s="13"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="18"/>
       <c r="G17" s="10">
         <v>45693</v>
       </c>
@@ -1180,12 +1182,12 @@
       <c r="AA17" s="2"/>
     </row>
     <row r="18" spans="1:62" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A18" s="19"/>
-      <c r="B18" s="19"/>
-      <c r="C18" s="19"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="15"/>
+      <c r="A18" s="21"/>
+      <c r="B18" s="21"/>
+      <c r="C18" s="21"/>
+      <c r="D18" s="19"/>
+      <c r="E18" s="19"/>
+      <c r="F18" s="20"/>
       <c r="G18" s="10">
         <v>45693</v>
       </c>
@@ -1193,16 +1195,16 @@
       <c r="AA18" s="2"/>
     </row>
     <row r="19" spans="1:62" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A19" s="19" t="s">
+      <c r="A19" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="B19" s="19"/>
-      <c r="C19" s="19"/>
-      <c r="D19" s="12">
+      <c r="B19" s="21"/>
+      <c r="C19" s="21"/>
+      <c r="D19" s="17">
         <v>2</v>
       </c>
-      <c r="E19" s="12"/>
-      <c r="F19" s="13"/>
+      <c r="E19" s="17"/>
+      <c r="F19" s="18"/>
       <c r="G19" s="10">
         <v>45693</v>
       </c>
@@ -1210,12 +1212,12 @@
       <c r="AA19" s="2"/>
     </row>
     <row r="20" spans="1:62" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A20" s="19"/>
-      <c r="B20" s="19"/>
-      <c r="C20" s="19"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14"/>
-      <c r="F20" s="15"/>
+      <c r="A20" s="21"/>
+      <c r="B20" s="21"/>
+      <c r="C20" s="21"/>
+      <c r="D20" s="19"/>
+      <c r="E20" s="19"/>
+      <c r="F20" s="20"/>
       <c r="G20" s="10">
         <v>45693</v>
       </c>
@@ -1223,16 +1225,16 @@
       <c r="AA20" s="2"/>
     </row>
     <row r="21" spans="1:62" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A21" s="18" t="s">
+      <c r="A21" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="B21" s="18"/>
-      <c r="C21" s="18"/>
-      <c r="D21" s="12">
+      <c r="B21" s="22"/>
+      <c r="C21" s="22"/>
+      <c r="D21" s="17">
         <v>6</v>
       </c>
-      <c r="E21" s="12"/>
-      <c r="F21" s="13"/>
+      <c r="E21" s="17"/>
+      <c r="F21" s="18"/>
       <c r="G21" s="10">
         <v>45700</v>
       </c>
@@ -1244,12 +1246,12 @@
       <c r="AG21" s="3"/>
     </row>
     <row r="22" spans="1:62" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A22" s="18"/>
-      <c r="B22" s="18"/>
-      <c r="C22" s="18"/>
-      <c r="D22" s="14"/>
-      <c r="E22" s="14"/>
-      <c r="F22" s="15"/>
+      <c r="A22" s="22"/>
+      <c r="B22" s="22"/>
+      <c r="C22" s="22"/>
+      <c r="D22" s="19"/>
+      <c r="E22" s="19"/>
+      <c r="F22" s="20"/>
       <c r="G22" s="10">
         <v>45714</v>
       </c>
@@ -1261,16 +1263,16 @@
       <c r="AG22" s="3"/>
     </row>
     <row r="23" spans="1:62" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A23" s="18" t="s">
+      <c r="A23" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="B23" s="18"/>
-      <c r="C23" s="18"/>
-      <c r="D23" s="12">
+      <c r="B23" s="22"/>
+      <c r="C23" s="22"/>
+      <c r="D23" s="17">
         <v>5</v>
       </c>
-      <c r="E23" s="12"/>
-      <c r="F23" s="13"/>
+      <c r="E23" s="17"/>
+      <c r="F23" s="18"/>
       <c r="G23" s="10">
         <v>45700</v>
       </c>
@@ -1285,12 +1287,12 @@
       <c r="AM23" s="7"/>
     </row>
     <row r="24" spans="1:62" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A24" s="18"/>
-      <c r="B24" s="18"/>
-      <c r="C24" s="18"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="14"/>
-      <c r="F24" s="15"/>
+      <c r="A24" s="22"/>
+      <c r="B24" s="22"/>
+      <c r="C24" s="22"/>
+      <c r="D24" s="19"/>
+      <c r="E24" s="19"/>
+      <c r="F24" s="20"/>
       <c r="G24" s="10">
         <v>45714</v>
       </c>
@@ -1305,18 +1307,18 @@
       <c r="AM24" s="7"/>
     </row>
     <row r="25" spans="1:62" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A25" s="18" t="s">
+      <c r="A25" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="B25" s="18"/>
-      <c r="C25" s="18"/>
-      <c r="D25" s="12">
-        <v>6</v>
-      </c>
-      <c r="E25" s="12"/>
-      <c r="F25" s="13"/>
+      <c r="B25" s="22"/>
+      <c r="C25" s="22"/>
+      <c r="D25" s="17">
+        <v>12</v>
+      </c>
+      <c r="E25" s="17"/>
+      <c r="F25" s="18"/>
       <c r="G25" s="10">
-        <v>45728</v>
+        <v>45721</v>
       </c>
       <c r="AE25" s="7"/>
       <c r="AF25" s="7"/>
@@ -1327,16 +1329,22 @@
       <c r="AP25" s="3"/>
       <c r="AQ25" s="3"/>
       <c r="AR25" s="3"/>
+      <c r="AS25" s="3"/>
+      <c r="AT25" s="3"/>
+      <c r="AU25" s="3"/>
+      <c r="AV25" s="3"/>
+      <c r="AW25" s="3"/>
+      <c r="AX25" s="3"/>
     </row>
     <row r="26" spans="1:62" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A26" s="18"/>
-      <c r="B26" s="18"/>
-      <c r="C26" s="18"/>
-      <c r="D26" s="14"/>
-      <c r="E26" s="14"/>
-      <c r="F26" s="15"/>
+      <c r="A26" s="22"/>
+      <c r="B26" s="22"/>
+      <c r="C26" s="22"/>
+      <c r="D26" s="19"/>
+      <c r="E26" s="19"/>
+      <c r="F26" s="20"/>
       <c r="G26" s="10">
-        <v>45735</v>
+        <v>45749</v>
       </c>
       <c r="AE26" s="7"/>
       <c r="AF26" s="7"/>
@@ -1347,18 +1355,24 @@
       <c r="AP26" s="3"/>
       <c r="AQ26" s="3"/>
       <c r="AR26" s="3"/>
+      <c r="AS26" s="3"/>
+      <c r="AT26" s="3"/>
+      <c r="AU26" s="3"/>
+      <c r="AV26" s="3"/>
+      <c r="AW26" s="3"/>
+      <c r="AX26" s="3"/>
     </row>
     <row r="27" spans="1:62" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A27" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="B27" s="18"/>
-      <c r="C27" s="18"/>
-      <c r="D27" s="12">
+      <c r="A27" s="22" t="s">
+        <v>23</v>
+      </c>
+      <c r="B27" s="22"/>
+      <c r="C27" s="22"/>
+      <c r="D27" s="17">
         <v>6</v>
       </c>
-      <c r="E27" s="12"/>
-      <c r="F27" s="13"/>
+      <c r="E27" s="17"/>
+      <c r="F27" s="18"/>
       <c r="G27" s="10">
         <v>45742</v>
       </c>
@@ -1374,14 +1388,15 @@
       <c r="AV27" s="3"/>
       <c r="AW27" s="3"/>
       <c r="AX27" s="3"/>
+      <c r="AY27" s="3"/>
     </row>
     <row r="28" spans="1:62" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A28" s="18"/>
-      <c r="B28" s="18"/>
-      <c r="C28" s="18"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="14"/>
-      <c r="F28" s="15"/>
+      <c r="A28" s="22"/>
+      <c r="B28" s="22"/>
+      <c r="C28" s="22"/>
+      <c r="D28" s="19"/>
+      <c r="E28" s="19"/>
+      <c r="F28" s="20"/>
       <c r="G28" s="10">
         <v>45749</v>
       </c>
@@ -1397,18 +1412,19 @@
       <c r="AV28" s="3"/>
       <c r="AW28" s="3"/>
       <c r="AX28" s="3"/>
+      <c r="AY28" s="3"/>
     </row>
     <row r="29" spans="1:62" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A29" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="B29" s="18"/>
-      <c r="C29" s="18"/>
-      <c r="D29" s="12">
+      <c r="A29" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="B29" s="22"/>
+      <c r="C29" s="22"/>
+      <c r="D29" s="17">
         <v>6</v>
       </c>
-      <c r="E29" s="12"/>
-      <c r="F29" s="13"/>
+      <c r="E29" s="17"/>
+      <c r="F29" s="18"/>
       <c r="G29" s="10">
         <v>45756</v>
       </c>
@@ -1429,12 +1445,12 @@
       <c r="BD29" s="3"/>
     </row>
     <row r="30" spans="1:62" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A30" s="18"/>
-      <c r="B30" s="18"/>
-      <c r="C30" s="18"/>
-      <c r="D30" s="14"/>
-      <c r="E30" s="14"/>
-      <c r="F30" s="15"/>
+      <c r="A30" s="22"/>
+      <c r="B30" s="22"/>
+      <c r="C30" s="22"/>
+      <c r="D30" s="19"/>
+      <c r="E30" s="19"/>
+      <c r="F30" s="20"/>
       <c r="G30" s="10">
         <v>45763</v>
       </c>
@@ -1449,16 +1465,16 @@
       <c r="BD30" s="3"/>
     </row>
     <row r="31" spans="1:62" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A31" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="B31" s="18"/>
-      <c r="C31" s="18"/>
-      <c r="D31" s="12">
+      <c r="A31" s="22" t="s">
+        <v>14</v>
+      </c>
+      <c r="B31" s="22"/>
+      <c r="C31" s="22"/>
+      <c r="D31" s="17">
         <v>6</v>
       </c>
-      <c r="E31" s="12"/>
-      <c r="F31" s="13"/>
+      <c r="E31" s="17"/>
+      <c r="F31" s="18"/>
       <c r="G31" s="10">
         <v>45777</v>
       </c>
@@ -1474,12 +1490,12 @@
       <c r="BJ31" s="3"/>
     </row>
     <row r="32" spans="1:62" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A32" s="18"/>
-      <c r="B32" s="18"/>
-      <c r="C32" s="18"/>
-      <c r="D32" s="14"/>
-      <c r="E32" s="14"/>
-      <c r="F32" s="15"/>
+      <c r="A32" s="22"/>
+      <c r="B32" s="22"/>
+      <c r="C32" s="22"/>
+      <c r="D32" s="19"/>
+      <c r="E32" s="19"/>
+      <c r="F32" s="20"/>
       <c r="G32" s="10">
         <v>45778</v>
       </c>
@@ -1495,16 +1511,16 @@
       <c r="BJ32" s="3"/>
     </row>
     <row r="33" spans="1:73" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A33" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="B33" s="17"/>
-      <c r="C33" s="17"/>
-      <c r="D33" s="12">
+      <c r="A33" s="23" t="s">
+        <v>15</v>
+      </c>
+      <c r="B33" s="23"/>
+      <c r="C33" s="23"/>
+      <c r="D33" s="17">
         <v>2</v>
       </c>
-      <c r="E33" s="12"/>
-      <c r="F33" s="13"/>
+      <c r="E33" s="17"/>
+      <c r="F33" s="18"/>
       <c r="G33" s="10">
         <v>45785</v>
       </c>
@@ -1512,12 +1528,12 @@
       <c r="BL33" s="4"/>
     </row>
     <row r="34" spans="1:73" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A34" s="17"/>
-      <c r="B34" s="17"/>
-      <c r="C34" s="17"/>
-      <c r="D34" s="14"/>
-      <c r="E34" s="14"/>
-      <c r="F34" s="15"/>
+      <c r="A34" s="23"/>
+      <c r="B34" s="23"/>
+      <c r="C34" s="23"/>
+      <c r="D34" s="19"/>
+      <c r="E34" s="19"/>
+      <c r="F34" s="20"/>
       <c r="G34" s="10">
         <v>45785</v>
       </c>
@@ -1525,16 +1541,16 @@
       <c r="BL34" s="4"/>
     </row>
     <row r="35" spans="1:73" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A35" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="B35" s="17"/>
-      <c r="C35" s="17"/>
-      <c r="D35" s="12">
+      <c r="A35" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="B35" s="23"/>
+      <c r="C35" s="23"/>
+      <c r="D35" s="17">
         <v>2</v>
       </c>
-      <c r="E35" s="12"/>
-      <c r="F35" s="13"/>
+      <c r="E35" s="17"/>
+      <c r="F35" s="18"/>
       <c r="G35" s="10">
         <v>45785</v>
       </c>
@@ -1542,12 +1558,12 @@
       <c r="BL35" s="4"/>
     </row>
     <row r="36" spans="1:73" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A36" s="17"/>
-      <c r="B36" s="17"/>
-      <c r="C36" s="17"/>
-      <c r="D36" s="14"/>
-      <c r="E36" s="14"/>
-      <c r="F36" s="15"/>
+      <c r="A36" s="23"/>
+      <c r="B36" s="23"/>
+      <c r="C36" s="23"/>
+      <c r="D36" s="19"/>
+      <c r="E36" s="19"/>
+      <c r="F36" s="20"/>
       <c r="G36" s="10">
         <v>45785</v>
       </c>
@@ -1555,16 +1571,16 @@
       <c r="BL36" s="4"/>
     </row>
     <row r="37" spans="1:73" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A37" s="17" t="s">
-        <v>17</v>
-      </c>
-      <c r="B37" s="17"/>
-      <c r="C37" s="17"/>
-      <c r="D37" s="12">
+      <c r="A37" s="23" t="s">
+        <v>16</v>
+      </c>
+      <c r="B37" s="23"/>
+      <c r="C37" s="23"/>
+      <c r="D37" s="17">
         <v>2</v>
       </c>
-      <c r="E37" s="12"/>
-      <c r="F37" s="13"/>
+      <c r="E37" s="17"/>
+      <c r="F37" s="18"/>
       <c r="G37" s="10">
         <v>45785</v>
       </c>
@@ -1572,12 +1588,12 @@
       <c r="BL37" s="4"/>
     </row>
     <row r="38" spans="1:73" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A38" s="17"/>
-      <c r="B38" s="17"/>
-      <c r="C38" s="17"/>
-      <c r="D38" s="14"/>
-      <c r="E38" s="14"/>
-      <c r="F38" s="15"/>
+      <c r="A38" s="23"/>
+      <c r="B38" s="23"/>
+      <c r="C38" s="23"/>
+      <c r="D38" s="19"/>
+      <c r="E38" s="19"/>
+      <c r="F38" s="20"/>
       <c r="G38" s="10">
         <v>45785</v>
       </c>
@@ -1585,16 +1601,16 @@
       <c r="BL38" s="4"/>
     </row>
     <row r="39" spans="1:73" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A39" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="B39" s="17"/>
-      <c r="C39" s="17"/>
-      <c r="D39" s="12">
+      <c r="A39" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="B39" s="23"/>
+      <c r="C39" s="23"/>
+      <c r="D39" s="17">
         <v>2</v>
       </c>
-      <c r="E39" s="12"/>
-      <c r="F39" s="13"/>
+      <c r="E39" s="17"/>
+      <c r="F39" s="18"/>
       <c r="G39" s="10">
         <v>45785</v>
       </c>
@@ -1602,12 +1618,12 @@
       <c r="BL39" s="4"/>
     </row>
     <row r="40" spans="1:73" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A40" s="17"/>
-      <c r="B40" s="17"/>
-      <c r="C40" s="17"/>
-      <c r="D40" s="14"/>
-      <c r="E40" s="14"/>
-      <c r="F40" s="15"/>
+      <c r="A40" s="23"/>
+      <c r="B40" s="23"/>
+      <c r="C40" s="23"/>
+      <c r="D40" s="19"/>
+      <c r="E40" s="19"/>
+      <c r="F40" s="20"/>
       <c r="G40" s="10">
         <v>45785</v>
       </c>
@@ -1615,16 +1631,16 @@
       <c r="BL40" s="4"/>
     </row>
     <row r="41" spans="1:73" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A41" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="B41" s="11"/>
-      <c r="C41" s="11"/>
-      <c r="D41" s="12">
+      <c r="A41" s="24" t="s">
+        <v>18</v>
+      </c>
+      <c r="B41" s="24"/>
+      <c r="C41" s="24"/>
+      <c r="D41" s="17">
         <v>4</v>
       </c>
-      <c r="E41" s="12"/>
-      <c r="F41" s="13"/>
+      <c r="E41" s="17"/>
+      <c r="F41" s="18"/>
       <c r="G41" s="10">
         <v>45792</v>
       </c>
@@ -1634,12 +1650,12 @@
       <c r="BP41" s="5"/>
     </row>
     <row r="42" spans="1:73" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A42" s="11"/>
-      <c r="B42" s="11"/>
-      <c r="C42" s="11"/>
-      <c r="D42" s="14"/>
-      <c r="E42" s="14"/>
-      <c r="F42" s="15"/>
+      <c r="A42" s="24"/>
+      <c r="B42" s="24"/>
+      <c r="C42" s="24"/>
+      <c r="D42" s="19"/>
+      <c r="E42" s="19"/>
+      <c r="F42" s="20"/>
       <c r="G42" s="10">
         <v>45792</v>
       </c>
@@ -1649,28 +1665,28 @@
       <c r="BP42" s="5"/>
     </row>
     <row r="43" spans="1:73" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A43" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="B43" s="16"/>
-      <c r="C43" s="16"/>
-      <c r="D43" s="12">
+      <c r="A43" s="25" t="s">
+        <v>19</v>
+      </c>
+      <c r="B43" s="25"/>
+      <c r="C43" s="25"/>
+      <c r="D43" s="17">
         <f>SUM(D3:F42)</f>
-        <v>68</v>
-      </c>
-      <c r="E43" s="12"/>
-      <c r="F43" s="13"/>
+        <v>74</v>
+      </c>
+      <c r="E43" s="17"/>
+      <c r="F43" s="18"/>
       <c r="G43" s="9">
         <v>45665</v>
       </c>
     </row>
     <row r="44" spans="1:73" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A44" s="16"/>
-      <c r="B44" s="16"/>
-      <c r="C44" s="16"/>
-      <c r="D44" s="14"/>
-      <c r="E44" s="14"/>
-      <c r="F44" s="15"/>
+      <c r="A44" s="25"/>
+      <c r="B44" s="25"/>
+      <c r="C44" s="25"/>
+      <c r="D44" s="19"/>
+      <c r="E44" s="19"/>
+      <c r="F44" s="20"/>
       <c r="G44" s="10">
         <v>45820</v>
       </c>
@@ -1742,17 +1758,17 @@
       <c r="BU44" s="7"/>
     </row>
     <row r="45" spans="1:73" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A45" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="B45" s="16"/>
-      <c r="C45" s="16"/>
-      <c r="D45" s="12">
+      <c r="A45" s="25" t="s">
+        <v>20</v>
+      </c>
+      <c r="B45" s="25"/>
+      <c r="C45" s="25"/>
+      <c r="D45" s="17">
         <f>SUM(D3:F42)</f>
-        <v>68</v>
-      </c>
-      <c r="E45" s="12"/>
-      <c r="F45" s="13"/>
+        <v>74</v>
+      </c>
+      <c r="E45" s="17"/>
+      <c r="F45" s="18"/>
       <c r="G45" s="9">
         <v>45665</v>
       </c>
@@ -1824,12 +1840,12 @@
       <c r="BU45" s="7"/>
     </row>
     <row r="46" spans="1:73" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A46" s="16"/>
-      <c r="B46" s="16"/>
-      <c r="C46" s="16"/>
-      <c r="D46" s="14"/>
-      <c r="E46" s="14"/>
-      <c r="F46" s="15"/>
+      <c r="A46" s="25"/>
+      <c r="B46" s="25"/>
+      <c r="C46" s="25"/>
+      <c r="D46" s="19"/>
+      <c r="E46" s="19"/>
+      <c r="F46" s="20"/>
       <c r="G46" s="10">
         <v>45820</v>
       </c>
@@ -1902,54 +1918,54 @@
     </row>
   </sheetData>
   <mergeCells count="48">
+    <mergeCell ref="A41:C42"/>
+    <mergeCell ref="D41:F42"/>
+    <mergeCell ref="A43:C44"/>
+    <mergeCell ref="D43:F44"/>
+    <mergeCell ref="A45:C46"/>
+    <mergeCell ref="D45:F46"/>
+    <mergeCell ref="A35:C36"/>
+    <mergeCell ref="D35:F36"/>
+    <mergeCell ref="A37:C38"/>
+    <mergeCell ref="D37:F38"/>
+    <mergeCell ref="A39:C40"/>
+    <mergeCell ref="D39:F40"/>
+    <mergeCell ref="A29:C30"/>
+    <mergeCell ref="D29:F30"/>
+    <mergeCell ref="A31:C32"/>
+    <mergeCell ref="D31:F32"/>
+    <mergeCell ref="A33:C34"/>
+    <mergeCell ref="D33:F34"/>
+    <mergeCell ref="A23:C24"/>
+    <mergeCell ref="D23:F24"/>
+    <mergeCell ref="A25:C26"/>
+    <mergeCell ref="D25:F26"/>
+    <mergeCell ref="A27:C28"/>
+    <mergeCell ref="D27:F28"/>
+    <mergeCell ref="A17:C18"/>
+    <mergeCell ref="D17:F18"/>
+    <mergeCell ref="A19:C20"/>
+    <mergeCell ref="D19:F20"/>
+    <mergeCell ref="A21:C22"/>
+    <mergeCell ref="D21:F22"/>
+    <mergeCell ref="A11:C12"/>
+    <mergeCell ref="D11:F12"/>
+    <mergeCell ref="A13:C14"/>
+    <mergeCell ref="D13:F14"/>
+    <mergeCell ref="A15:C16"/>
+    <mergeCell ref="D15:F16"/>
+    <mergeCell ref="A5:C6"/>
+    <mergeCell ref="D5:F6"/>
+    <mergeCell ref="A7:C8"/>
+    <mergeCell ref="D7:F8"/>
+    <mergeCell ref="A9:C10"/>
+    <mergeCell ref="D9:F10"/>
     <mergeCell ref="BD1:CZ2"/>
     <mergeCell ref="A1:C2"/>
     <mergeCell ref="D1:F2"/>
     <mergeCell ref="G1:BC2"/>
     <mergeCell ref="A3:C4"/>
     <mergeCell ref="D3:F4"/>
-    <mergeCell ref="A5:C6"/>
-    <mergeCell ref="D5:F6"/>
-    <mergeCell ref="A7:C8"/>
-    <mergeCell ref="D7:F8"/>
-    <mergeCell ref="A9:C10"/>
-    <mergeCell ref="D9:F10"/>
-    <mergeCell ref="A11:C12"/>
-    <mergeCell ref="D11:F12"/>
-    <mergeCell ref="A13:C14"/>
-    <mergeCell ref="D13:F14"/>
-    <mergeCell ref="A15:C16"/>
-    <mergeCell ref="D15:F16"/>
-    <mergeCell ref="A17:C18"/>
-    <mergeCell ref="D17:F18"/>
-    <mergeCell ref="A19:C20"/>
-    <mergeCell ref="D19:F20"/>
-    <mergeCell ref="A21:C22"/>
-    <mergeCell ref="D21:F22"/>
-    <mergeCell ref="A23:C24"/>
-    <mergeCell ref="D23:F24"/>
-    <mergeCell ref="A25:C26"/>
-    <mergeCell ref="D25:F26"/>
-    <mergeCell ref="A27:C28"/>
-    <mergeCell ref="D27:F28"/>
-    <mergeCell ref="A29:C30"/>
-    <mergeCell ref="D29:F30"/>
-    <mergeCell ref="A31:C32"/>
-    <mergeCell ref="D31:F32"/>
-    <mergeCell ref="A33:C34"/>
-    <mergeCell ref="D33:F34"/>
-    <mergeCell ref="A35:C36"/>
-    <mergeCell ref="D35:F36"/>
-    <mergeCell ref="A37:C38"/>
-    <mergeCell ref="D37:F38"/>
-    <mergeCell ref="A39:C40"/>
-    <mergeCell ref="D39:F40"/>
-    <mergeCell ref="A41:C42"/>
-    <mergeCell ref="D41:F42"/>
-    <mergeCell ref="A43:C44"/>
-    <mergeCell ref="D43:F44"/>
-    <mergeCell ref="A45:C46"/>
-    <mergeCell ref="D45:F46"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
commit mattutino, giornata sprint, aggiunto lavoro svolto pol a caasa
</commit_message>
<xml_diff>
--- a/7_Allegati/Gantt/Gantt_cons.xlsx
+++ b/7_Allegati/Gantt/Gantt_cons.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\M306\Progetto_CasaNote\7_Allegati\Gantt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FE9F9E8-6133-4894-AB29-C787D0D9FB9A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C69179E-478B-4287-910D-879248403ABD}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="14025" xr2:uid="{285B56FD-1A67-4790-99DC-B99A42CD0DBC}"/>
   </bookViews>
@@ -359,8 +359,23 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -374,35 +389,20 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -731,232 +731,232 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:104" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24" t="s">
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
-      <c r="K1" s="23"/>
-      <c r="L1" s="23"/>
-      <c r="M1" s="23"/>
-      <c r="N1" s="23"/>
-      <c r="O1" s="23"/>
-      <c r="P1" s="23"/>
-      <c r="Q1" s="23"/>
-      <c r="R1" s="23"/>
-      <c r="S1" s="23"/>
-      <c r="T1" s="23"/>
-      <c r="U1" s="23"/>
-      <c r="V1" s="23"/>
-      <c r="W1" s="23"/>
-      <c r="X1" s="23"/>
-      <c r="Y1" s="23"/>
-      <c r="Z1" s="23"/>
-      <c r="AA1" s="23"/>
-      <c r="AB1" s="23"/>
-      <c r="AC1" s="23"/>
-      <c r="AD1" s="23"/>
-      <c r="AE1" s="23"/>
-      <c r="AF1" s="23"/>
-      <c r="AG1" s="23"/>
-      <c r="AH1" s="23"/>
-      <c r="AI1" s="23"/>
-      <c r="AJ1" s="23"/>
-      <c r="AK1" s="23"/>
-      <c r="AL1" s="23"/>
-      <c r="AM1" s="23"/>
-      <c r="AN1" s="23"/>
-      <c r="AO1" s="23"/>
-      <c r="AP1" s="23"/>
-      <c r="AQ1" s="23"/>
-      <c r="AR1" s="23"/>
-      <c r="AS1" s="23"/>
-      <c r="AT1" s="23"/>
-      <c r="AU1" s="23"/>
-      <c r="AV1" s="23"/>
-      <c r="AW1" s="23"/>
-      <c r="AX1" s="23"/>
-      <c r="AY1" s="23"/>
-      <c r="AZ1" s="23"/>
-      <c r="BA1" s="23"/>
-      <c r="BB1" s="23"/>
-      <c r="BC1" s="23"/>
-      <c r="BD1" s="23"/>
-      <c r="BE1" s="23"/>
-      <c r="BF1" s="23"/>
-      <c r="BG1" s="23"/>
-      <c r="BH1" s="23"/>
-      <c r="BI1" s="23"/>
-      <c r="BJ1" s="23"/>
-      <c r="BK1" s="23"/>
-      <c r="BL1" s="23"/>
-      <c r="BM1" s="23"/>
-      <c r="BN1" s="23"/>
-      <c r="BO1" s="23"/>
-      <c r="BP1" s="23"/>
-      <c r="BQ1" s="23"/>
-      <c r="BR1" s="23"/>
-      <c r="BS1" s="23"/>
-      <c r="BT1" s="23"/>
-      <c r="BU1" s="23"/>
-      <c r="BV1" s="23"/>
-      <c r="BW1" s="23"/>
-      <c r="BX1" s="23"/>
-      <c r="BY1" s="23"/>
-      <c r="BZ1" s="23"/>
-      <c r="CA1" s="23"/>
-      <c r="CB1" s="23"/>
-      <c r="CC1" s="23"/>
-      <c r="CD1" s="23"/>
-      <c r="CE1" s="23"/>
-      <c r="CF1" s="23"/>
-      <c r="CG1" s="23"/>
-      <c r="CH1" s="23"/>
-      <c r="CI1" s="23"/>
-      <c r="CJ1" s="23"/>
-      <c r="CK1" s="23"/>
-      <c r="CL1" s="23"/>
-      <c r="CM1" s="23"/>
-      <c r="CN1" s="23"/>
-      <c r="CO1" s="23"/>
-      <c r="CP1" s="23"/>
-      <c r="CQ1" s="23"/>
-      <c r="CR1" s="23"/>
-      <c r="CS1" s="23"/>
-      <c r="CT1" s="23"/>
-      <c r="CU1" s="23"/>
-      <c r="CV1" s="23"/>
-      <c r="CW1" s="23"/>
-      <c r="CX1" s="23"/>
-      <c r="CY1" s="23"/>
-      <c r="CZ1" s="23"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
+      <c r="J1" s="11"/>
+      <c r="K1" s="11"/>
+      <c r="L1" s="11"/>
+      <c r="M1" s="11"/>
+      <c r="N1" s="11"/>
+      <c r="O1" s="11"/>
+      <c r="P1" s="11"/>
+      <c r="Q1" s="11"/>
+      <c r="R1" s="11"/>
+      <c r="S1" s="11"/>
+      <c r="T1" s="11"/>
+      <c r="U1" s="11"/>
+      <c r="V1" s="11"/>
+      <c r="W1" s="11"/>
+      <c r="X1" s="11"/>
+      <c r="Y1" s="11"/>
+      <c r="Z1" s="11"/>
+      <c r="AA1" s="11"/>
+      <c r="AB1" s="11"/>
+      <c r="AC1" s="11"/>
+      <c r="AD1" s="11"/>
+      <c r="AE1" s="11"/>
+      <c r="AF1" s="11"/>
+      <c r="AG1" s="11"/>
+      <c r="AH1" s="11"/>
+      <c r="AI1" s="11"/>
+      <c r="AJ1" s="11"/>
+      <c r="AK1" s="11"/>
+      <c r="AL1" s="11"/>
+      <c r="AM1" s="11"/>
+      <c r="AN1" s="11"/>
+      <c r="AO1" s="11"/>
+      <c r="AP1" s="11"/>
+      <c r="AQ1" s="11"/>
+      <c r="AR1" s="11"/>
+      <c r="AS1" s="11"/>
+      <c r="AT1" s="11"/>
+      <c r="AU1" s="11"/>
+      <c r="AV1" s="11"/>
+      <c r="AW1" s="11"/>
+      <c r="AX1" s="11"/>
+      <c r="AY1" s="11"/>
+      <c r="AZ1" s="11"/>
+      <c r="BA1" s="11"/>
+      <c r="BB1" s="11"/>
+      <c r="BC1" s="11"/>
+      <c r="BD1" s="11"/>
+      <c r="BE1" s="11"/>
+      <c r="BF1" s="11"/>
+      <c r="BG1" s="11"/>
+      <c r="BH1" s="11"/>
+      <c r="BI1" s="11"/>
+      <c r="BJ1" s="11"/>
+      <c r="BK1" s="11"/>
+      <c r="BL1" s="11"/>
+      <c r="BM1" s="11"/>
+      <c r="BN1" s="11"/>
+      <c r="BO1" s="11"/>
+      <c r="BP1" s="11"/>
+      <c r="BQ1" s="11"/>
+      <c r="BR1" s="11"/>
+      <c r="BS1" s="11"/>
+      <c r="BT1" s="11"/>
+      <c r="BU1" s="11"/>
+      <c r="BV1" s="11"/>
+      <c r="BW1" s="11"/>
+      <c r="BX1" s="11"/>
+      <c r="BY1" s="11"/>
+      <c r="BZ1" s="11"/>
+      <c r="CA1" s="11"/>
+      <c r="CB1" s="11"/>
+      <c r="CC1" s="11"/>
+      <c r="CD1" s="11"/>
+      <c r="CE1" s="11"/>
+      <c r="CF1" s="11"/>
+      <c r="CG1" s="11"/>
+      <c r="CH1" s="11"/>
+      <c r="CI1" s="11"/>
+      <c r="CJ1" s="11"/>
+      <c r="CK1" s="11"/>
+      <c r="CL1" s="11"/>
+      <c r="CM1" s="11"/>
+      <c r="CN1" s="11"/>
+      <c r="CO1" s="11"/>
+      <c r="CP1" s="11"/>
+      <c r="CQ1" s="11"/>
+      <c r="CR1" s="11"/>
+      <c r="CS1" s="11"/>
+      <c r="CT1" s="11"/>
+      <c r="CU1" s="11"/>
+      <c r="CV1" s="11"/>
+      <c r="CW1" s="11"/>
+      <c r="CX1" s="11"/>
+      <c r="CY1" s="11"/>
+      <c r="CZ1" s="11"/>
     </row>
     <row r="2" spans="1:104" ht="16.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="25"/>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
-      <c r="I2" s="23"/>
-      <c r="J2" s="23"/>
-      <c r="K2" s="23"/>
-      <c r="L2" s="23"/>
-      <c r="M2" s="23"/>
-      <c r="N2" s="23"/>
-      <c r="O2" s="23"/>
-      <c r="P2" s="23"/>
-      <c r="Q2" s="23"/>
-      <c r="R2" s="23"/>
-      <c r="S2" s="23"/>
-      <c r="T2" s="23"/>
-      <c r="U2" s="23"/>
-      <c r="V2" s="23"/>
-      <c r="W2" s="23"/>
-      <c r="X2" s="23"/>
-      <c r="Y2" s="23"/>
-      <c r="Z2" s="23"/>
-      <c r="AA2" s="23"/>
-      <c r="AB2" s="23"/>
-      <c r="AC2" s="23"/>
-      <c r="AD2" s="23"/>
-      <c r="AE2" s="23"/>
-      <c r="AF2" s="23"/>
-      <c r="AG2" s="23"/>
-      <c r="AH2" s="23"/>
-      <c r="AI2" s="23"/>
-      <c r="AJ2" s="23"/>
-      <c r="AK2" s="23"/>
-      <c r="AL2" s="23"/>
-      <c r="AM2" s="23"/>
-      <c r="AN2" s="23"/>
-      <c r="AO2" s="23"/>
-      <c r="AP2" s="23"/>
-      <c r="AQ2" s="23"/>
-      <c r="AR2" s="23"/>
-      <c r="AS2" s="23"/>
-      <c r="AT2" s="23"/>
-      <c r="AU2" s="23"/>
-      <c r="AV2" s="23"/>
-      <c r="AW2" s="23"/>
-      <c r="AX2" s="23"/>
-      <c r="AY2" s="23"/>
-      <c r="AZ2" s="23"/>
-      <c r="BA2" s="23"/>
-      <c r="BB2" s="23"/>
-      <c r="BC2" s="23"/>
-      <c r="BD2" s="23"/>
-      <c r="BE2" s="23"/>
-      <c r="BF2" s="23"/>
-      <c r="BG2" s="23"/>
-      <c r="BH2" s="23"/>
-      <c r="BI2" s="23"/>
-      <c r="BJ2" s="23"/>
-      <c r="BK2" s="23"/>
-      <c r="BL2" s="23"/>
-      <c r="BM2" s="23"/>
-      <c r="BN2" s="23"/>
-      <c r="BO2" s="23"/>
-      <c r="BP2" s="23"/>
-      <c r="BQ2" s="23"/>
-      <c r="BR2" s="23"/>
-      <c r="BS2" s="23"/>
-      <c r="BT2" s="23"/>
-      <c r="BU2" s="23"/>
-      <c r="BV2" s="23"/>
-      <c r="BW2" s="23"/>
-      <c r="BX2" s="23"/>
-      <c r="BY2" s="23"/>
-      <c r="BZ2" s="23"/>
-      <c r="CA2" s="23"/>
-      <c r="CB2" s="23"/>
-      <c r="CC2" s="23"/>
-      <c r="CD2" s="23"/>
-      <c r="CE2" s="23"/>
-      <c r="CF2" s="23"/>
-      <c r="CG2" s="23"/>
-      <c r="CH2" s="23"/>
-      <c r="CI2" s="23"/>
-      <c r="CJ2" s="23"/>
-      <c r="CK2" s="23"/>
-      <c r="CL2" s="23"/>
-      <c r="CM2" s="23"/>
-      <c r="CN2" s="23"/>
-      <c r="CO2" s="23"/>
-      <c r="CP2" s="23"/>
-      <c r="CQ2" s="23"/>
-      <c r="CR2" s="23"/>
-      <c r="CS2" s="23"/>
-      <c r="CT2" s="23"/>
-      <c r="CU2" s="23"/>
-      <c r="CV2" s="23"/>
-      <c r="CW2" s="23"/>
-      <c r="CX2" s="23"/>
-      <c r="CY2" s="23"/>
-      <c r="CZ2" s="23"/>
+      <c r="A2" s="13"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="11"/>
+      <c r="H2" s="11"/>
+      <c r="I2" s="11"/>
+      <c r="J2" s="11"/>
+      <c r="K2" s="11"/>
+      <c r="L2" s="11"/>
+      <c r="M2" s="11"/>
+      <c r="N2" s="11"/>
+      <c r="O2" s="11"/>
+      <c r="P2" s="11"/>
+      <c r="Q2" s="11"/>
+      <c r="R2" s="11"/>
+      <c r="S2" s="11"/>
+      <c r="T2" s="11"/>
+      <c r="U2" s="11"/>
+      <c r="V2" s="11"/>
+      <c r="W2" s="11"/>
+      <c r="X2" s="11"/>
+      <c r="Y2" s="11"/>
+      <c r="Z2" s="11"/>
+      <c r="AA2" s="11"/>
+      <c r="AB2" s="11"/>
+      <c r="AC2" s="11"/>
+      <c r="AD2" s="11"/>
+      <c r="AE2" s="11"/>
+      <c r="AF2" s="11"/>
+      <c r="AG2" s="11"/>
+      <c r="AH2" s="11"/>
+      <c r="AI2" s="11"/>
+      <c r="AJ2" s="11"/>
+      <c r="AK2" s="11"/>
+      <c r="AL2" s="11"/>
+      <c r="AM2" s="11"/>
+      <c r="AN2" s="11"/>
+      <c r="AO2" s="11"/>
+      <c r="AP2" s="11"/>
+      <c r="AQ2" s="11"/>
+      <c r="AR2" s="11"/>
+      <c r="AS2" s="11"/>
+      <c r="AT2" s="11"/>
+      <c r="AU2" s="11"/>
+      <c r="AV2" s="11"/>
+      <c r="AW2" s="11"/>
+      <c r="AX2" s="11"/>
+      <c r="AY2" s="11"/>
+      <c r="AZ2" s="11"/>
+      <c r="BA2" s="11"/>
+      <c r="BB2" s="11"/>
+      <c r="BC2" s="11"/>
+      <c r="BD2" s="11"/>
+      <c r="BE2" s="11"/>
+      <c r="BF2" s="11"/>
+      <c r="BG2" s="11"/>
+      <c r="BH2" s="11"/>
+      <c r="BI2" s="11"/>
+      <c r="BJ2" s="11"/>
+      <c r="BK2" s="11"/>
+      <c r="BL2" s="11"/>
+      <c r="BM2" s="11"/>
+      <c r="BN2" s="11"/>
+      <c r="BO2" s="11"/>
+      <c r="BP2" s="11"/>
+      <c r="BQ2" s="11"/>
+      <c r="BR2" s="11"/>
+      <c r="BS2" s="11"/>
+      <c r="BT2" s="11"/>
+      <c r="BU2" s="11"/>
+      <c r="BV2" s="11"/>
+      <c r="BW2" s="11"/>
+      <c r="BX2" s="11"/>
+      <c r="BY2" s="11"/>
+      <c r="BZ2" s="11"/>
+      <c r="CA2" s="11"/>
+      <c r="CB2" s="11"/>
+      <c r="CC2" s="11"/>
+      <c r="CD2" s="11"/>
+      <c r="CE2" s="11"/>
+      <c r="CF2" s="11"/>
+      <c r="CG2" s="11"/>
+      <c r="CH2" s="11"/>
+      <c r="CI2" s="11"/>
+      <c r="CJ2" s="11"/>
+      <c r="CK2" s="11"/>
+      <c r="CL2" s="11"/>
+      <c r="CM2" s="11"/>
+      <c r="CN2" s="11"/>
+      <c r="CO2" s="11"/>
+      <c r="CP2" s="11"/>
+      <c r="CQ2" s="11"/>
+      <c r="CR2" s="11"/>
+      <c r="CS2" s="11"/>
+      <c r="CT2" s="11"/>
+      <c r="CU2" s="11"/>
+      <c r="CV2" s="11"/>
+      <c r="CW2" s="11"/>
+      <c r="CX2" s="11"/>
+      <c r="CY2" s="11"/>
+      <c r="CZ2" s="11"/>
     </row>
     <row r="3" spans="1:104" ht="29.25" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="21">
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="15">
         <v>3</v>
       </c>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="16"/>
       <c r="G3" s="8">
         <v>45665</v>
       </c>
@@ -965,12 +965,12 @@
       <c r="J3" s="1"/>
     </row>
     <row r="4" spans="1:104" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A4" s="20"/>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
+      <c r="A4" s="14"/>
+      <c r="B4" s="14"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="16"/>
       <c r="G4" s="9">
         <v>45665</v>
       </c>
@@ -979,16 +979,16 @@
       <c r="J4" s="1"/>
     </row>
     <row r="5" spans="1:104" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="20" t="s">
+      <c r="A5" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="20"/>
-      <c r="C5" s="20"/>
-      <c r="D5" s="21">
+      <c r="B5" s="14"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="15">
         <v>3</v>
       </c>
-      <c r="E5" s="22"/>
-      <c r="F5" s="22"/>
+      <c r="E5" s="16"/>
+      <c r="F5" s="16"/>
       <c r="G5" s="9">
         <v>45665</v>
       </c>
@@ -997,12 +997,12 @@
       <c r="M5" s="1"/>
     </row>
     <row r="6" spans="1:104" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A6" s="20"/>
-      <c r="B6" s="20"/>
-      <c r="C6" s="20"/>
-      <c r="D6" s="21"/>
-      <c r="E6" s="22"/>
-      <c r="F6" s="22"/>
+      <c r="A6" s="14"/>
+      <c r="B6" s="14"/>
+      <c r="C6" s="14"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="16"/>
       <c r="G6" s="9">
         <v>45665</v>
       </c>
@@ -1011,16 +1011,16 @@
       <c r="M6" s="1"/>
     </row>
     <row r="7" spans="1:104" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A7" s="20" t="s">
+      <c r="A7" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="20"/>
-      <c r="C7" s="20"/>
-      <c r="D7" s="12">
+      <c r="B7" s="14"/>
+      <c r="C7" s="14"/>
+      <c r="D7" s="17">
         <v>3</v>
       </c>
-      <c r="E7" s="12"/>
-      <c r="F7" s="13"/>
+      <c r="E7" s="17"/>
+      <c r="F7" s="18"/>
       <c r="G7" s="10">
         <v>45665</v>
       </c>
@@ -1029,12 +1029,12 @@
       <c r="P7" s="1"/>
     </row>
     <row r="8" spans="1:104" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A8" s="20"/>
-      <c r="B8" s="20"/>
-      <c r="C8" s="20"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="15"/>
+      <c r="A8" s="14"/>
+      <c r="B8" s="14"/>
+      <c r="C8" s="14"/>
+      <c r="D8" s="19"/>
+      <c r="E8" s="19"/>
+      <c r="F8" s="20"/>
       <c r="G8" s="10">
         <v>45672</v>
       </c>
@@ -1043,16 +1043,16 @@
       <c r="P8" s="1"/>
     </row>
     <row r="9" spans="1:104" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="19"/>
-      <c r="C9" s="19"/>
-      <c r="D9" s="12">
+      <c r="B9" s="21"/>
+      <c r="C9" s="21"/>
+      <c r="D9" s="17">
         <v>2</v>
       </c>
-      <c r="E9" s="12"/>
-      <c r="F9" s="13"/>
+      <c r="E9" s="17"/>
+      <c r="F9" s="18"/>
       <c r="G9" s="9">
         <v>45672</v>
       </c>
@@ -1061,12 +1061,12 @@
       <c r="S9" s="2"/>
     </row>
     <row r="10" spans="1:104" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A10" s="19"/>
-      <c r="B10" s="19"/>
-      <c r="C10" s="19"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="14"/>
-      <c r="F10" s="15"/>
+      <c r="A10" s="21"/>
+      <c r="B10" s="21"/>
+      <c r="C10" s="21"/>
+      <c r="D10" s="19"/>
+      <c r="E10" s="19"/>
+      <c r="F10" s="20"/>
       <c r="G10" s="9">
         <v>45679</v>
       </c>
@@ -1075,16 +1075,16 @@
       <c r="S10" s="2"/>
     </row>
     <row r="11" spans="1:104" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="B11" s="19"/>
-      <c r="C11" s="19"/>
-      <c r="D11" s="12">
+      <c r="B11" s="21"/>
+      <c r="C11" s="21"/>
+      <c r="D11" s="17">
         <v>2</v>
       </c>
-      <c r="E11" s="12"/>
-      <c r="F11" s="13"/>
+      <c r="E11" s="17"/>
+      <c r="F11" s="18"/>
       <c r="G11" s="9">
         <v>45672</v>
       </c>
@@ -1092,12 +1092,12 @@
       <c r="U11" s="2"/>
     </row>
     <row r="12" spans="1:104" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A12" s="19"/>
-      <c r="B12" s="19"/>
-      <c r="C12" s="19"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="15"/>
+      <c r="A12" s="21"/>
+      <c r="B12" s="21"/>
+      <c r="C12" s="21"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="20"/>
       <c r="G12" s="9">
         <v>45679</v>
       </c>
@@ -1105,16 +1105,16 @@
       <c r="U12" s="2"/>
     </row>
     <row r="13" spans="1:104" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A13" s="19" t="s">
+      <c r="A13" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="B13" s="19"/>
-      <c r="C13" s="19"/>
-      <c r="D13" s="12">
+      <c r="B13" s="21"/>
+      <c r="C13" s="21"/>
+      <c r="D13" s="17">
         <v>2</v>
       </c>
-      <c r="E13" s="12"/>
-      <c r="F13" s="13"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="18"/>
       <c r="G13" s="9">
         <v>45672</v>
       </c>
@@ -1122,12 +1122,12 @@
       <c r="W13" s="2"/>
     </row>
     <row r="14" spans="1:104" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A14" s="19"/>
-      <c r="B14" s="19"/>
-      <c r="C14" s="19"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="15"/>
+      <c r="A14" s="21"/>
+      <c r="B14" s="21"/>
+      <c r="C14" s="21"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="20"/>
       <c r="G14" s="9">
         <v>45679</v>
       </c>
@@ -1135,16 +1135,16 @@
       <c r="W14" s="2"/>
     </row>
     <row r="15" spans="1:104" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A15" s="19" t="s">
+      <c r="A15" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="B15" s="19"/>
-      <c r="C15" s="19"/>
-      <c r="D15" s="12">
+      <c r="B15" s="21"/>
+      <c r="C15" s="21"/>
+      <c r="D15" s="17">
         <v>2</v>
       </c>
-      <c r="E15" s="12"/>
-      <c r="F15" s="13"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="18"/>
       <c r="G15" s="9">
         <v>45679</v>
       </c>
@@ -1152,12 +1152,12 @@
       <c r="Y15" s="2"/>
     </row>
     <row r="16" spans="1:104" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A16" s="19"/>
-      <c r="B16" s="19"/>
-      <c r="C16" s="19"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14"/>
-      <c r="F16" s="15"/>
+      <c r="A16" s="21"/>
+      <c r="B16" s="21"/>
+      <c r="C16" s="21"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="20"/>
       <c r="G16" s="10">
         <v>45693</v>
       </c>
@@ -1165,16 +1165,16 @@
       <c r="Y16" s="2"/>
     </row>
     <row r="17" spans="1:62" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A17" s="19" t="s">
+      <c r="A17" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="B17" s="19"/>
-      <c r="C17" s="19"/>
-      <c r="D17" s="12">
+      <c r="B17" s="21"/>
+      <c r="C17" s="21"/>
+      <c r="D17" s="17">
         <v>2</v>
       </c>
-      <c r="E17" s="12"/>
-      <c r="F17" s="13"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="18"/>
       <c r="G17" s="10">
         <v>45693</v>
       </c>
@@ -1182,12 +1182,12 @@
       <c r="AA17" s="2"/>
     </row>
     <row r="18" spans="1:62" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A18" s="19"/>
-      <c r="B18" s="19"/>
-      <c r="C18" s="19"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="15"/>
+      <c r="A18" s="21"/>
+      <c r="B18" s="21"/>
+      <c r="C18" s="21"/>
+      <c r="D18" s="19"/>
+      <c r="E18" s="19"/>
+      <c r="F18" s="20"/>
       <c r="G18" s="10">
         <v>45693</v>
       </c>
@@ -1195,16 +1195,16 @@
       <c r="AA18" s="2"/>
     </row>
     <row r="19" spans="1:62" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A19" s="19" t="s">
+      <c r="A19" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="B19" s="19"/>
-      <c r="C19" s="19"/>
-      <c r="D19" s="12">
+      <c r="B19" s="21"/>
+      <c r="C19" s="21"/>
+      <c r="D19" s="17">
         <v>2</v>
       </c>
-      <c r="E19" s="12"/>
-      <c r="F19" s="13"/>
+      <c r="E19" s="17"/>
+      <c r="F19" s="18"/>
       <c r="G19" s="10">
         <v>45693</v>
       </c>
@@ -1212,12 +1212,12 @@
       <c r="AA19" s="2"/>
     </row>
     <row r="20" spans="1:62" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A20" s="19"/>
-      <c r="B20" s="19"/>
-      <c r="C20" s="19"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14"/>
-      <c r="F20" s="15"/>
+      <c r="A20" s="21"/>
+      <c r="B20" s="21"/>
+      <c r="C20" s="21"/>
+      <c r="D20" s="19"/>
+      <c r="E20" s="19"/>
+      <c r="F20" s="20"/>
       <c r="G20" s="10">
         <v>45693</v>
       </c>
@@ -1225,16 +1225,16 @@
       <c r="AA20" s="2"/>
     </row>
     <row r="21" spans="1:62" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A21" s="18" t="s">
+      <c r="A21" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="B21" s="18"/>
-      <c r="C21" s="18"/>
-      <c r="D21" s="12">
+      <c r="B21" s="22"/>
+      <c r="C21" s="22"/>
+      <c r="D21" s="17">
         <v>6</v>
       </c>
-      <c r="E21" s="12"/>
-      <c r="F21" s="13"/>
+      <c r="E21" s="17"/>
+      <c r="F21" s="18"/>
       <c r="G21" s="10">
         <v>45700</v>
       </c>
@@ -1246,12 +1246,12 @@
       <c r="AG21" s="3"/>
     </row>
     <row r="22" spans="1:62" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A22" s="18"/>
-      <c r="B22" s="18"/>
-      <c r="C22" s="18"/>
-      <c r="D22" s="14"/>
-      <c r="E22" s="14"/>
-      <c r="F22" s="15"/>
+      <c r="A22" s="22"/>
+      <c r="B22" s="22"/>
+      <c r="C22" s="22"/>
+      <c r="D22" s="19"/>
+      <c r="E22" s="19"/>
+      <c r="F22" s="20"/>
       <c r="G22" s="10">
         <v>45714</v>
       </c>
@@ -1263,16 +1263,16 @@
       <c r="AG22" s="3"/>
     </row>
     <row r="23" spans="1:62" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A23" s="18" t="s">
+      <c r="A23" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="B23" s="18"/>
-      <c r="C23" s="18"/>
-      <c r="D23" s="12">
+      <c r="B23" s="22"/>
+      <c r="C23" s="22"/>
+      <c r="D23" s="17">
         <v>5</v>
       </c>
-      <c r="E23" s="12"/>
-      <c r="F23" s="13"/>
+      <c r="E23" s="17"/>
+      <c r="F23" s="18"/>
       <c r="G23" s="10">
         <v>45700</v>
       </c>
@@ -1287,12 +1287,12 @@
       <c r="AM23" s="7"/>
     </row>
     <row r="24" spans="1:62" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A24" s="18"/>
-      <c r="B24" s="18"/>
-      <c r="C24" s="18"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="14"/>
-      <c r="F24" s="15"/>
+      <c r="A24" s="22"/>
+      <c r="B24" s="22"/>
+      <c r="C24" s="22"/>
+      <c r="D24" s="19"/>
+      <c r="E24" s="19"/>
+      <c r="F24" s="20"/>
       <c r="G24" s="10">
         <v>45714</v>
       </c>
@@ -1307,16 +1307,16 @@
       <c r="AM24" s="7"/>
     </row>
     <row r="25" spans="1:62" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A25" s="18" t="s">
+      <c r="A25" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="B25" s="18"/>
-      <c r="C25" s="18"/>
-      <c r="D25" s="12">
+      <c r="B25" s="22"/>
+      <c r="C25" s="22"/>
+      <c r="D25" s="17">
         <v>12</v>
       </c>
-      <c r="E25" s="12"/>
-      <c r="F25" s="13"/>
+      <c r="E25" s="17"/>
+      <c r="F25" s="18"/>
       <c r="G25" s="10">
         <v>45721</v>
       </c>
@@ -1337,12 +1337,12 @@
       <c r="AX25" s="3"/>
     </row>
     <row r="26" spans="1:62" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A26" s="18"/>
-      <c r="B26" s="18"/>
-      <c r="C26" s="18"/>
-      <c r="D26" s="14"/>
-      <c r="E26" s="14"/>
-      <c r="F26" s="15"/>
+      <c r="A26" s="22"/>
+      <c r="B26" s="22"/>
+      <c r="C26" s="22"/>
+      <c r="D26" s="19"/>
+      <c r="E26" s="19"/>
+      <c r="F26" s="20"/>
       <c r="G26" s="10">
         <v>45749</v>
       </c>
@@ -1363,16 +1363,16 @@
       <c r="AX26" s="3"/>
     </row>
     <row r="27" spans="1:62" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A27" s="18" t="s">
+      <c r="A27" s="22" t="s">
         <v>23</v>
       </c>
-      <c r="B27" s="18"/>
-      <c r="C27" s="18"/>
-      <c r="D27" s="12">
-        <v>6</v>
-      </c>
-      <c r="E27" s="12"/>
-      <c r="F27" s="13"/>
+      <c r="B27" s="22"/>
+      <c r="C27" s="22"/>
+      <c r="D27" s="17">
+        <v>10</v>
+      </c>
+      <c r="E27" s="17"/>
+      <c r="F27" s="18"/>
       <c r="G27" s="10">
         <v>45742</v>
       </c>
@@ -1389,14 +1389,17 @@
       <c r="AW27" s="3"/>
       <c r="AX27" s="3"/>
       <c r="AY27" s="3"/>
+      <c r="AZ27" s="3"/>
+      <c r="BA27" s="3"/>
+      <c r="BB27" s="3"/>
     </row>
     <row r="28" spans="1:62" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A28" s="18"/>
-      <c r="B28" s="18"/>
-      <c r="C28" s="18"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="14"/>
-      <c r="F28" s="15"/>
+      <c r="A28" s="22"/>
+      <c r="B28" s="22"/>
+      <c r="C28" s="22"/>
+      <c r="D28" s="19"/>
+      <c r="E28" s="19"/>
+      <c r="F28" s="20"/>
       <c r="G28" s="10">
         <v>45749</v>
       </c>
@@ -1413,20 +1416,23 @@
       <c r="AW28" s="3"/>
       <c r="AX28" s="3"/>
       <c r="AY28" s="3"/>
+      <c r="AZ28" s="3"/>
+      <c r="BA28" s="3"/>
+      <c r="BB28" s="3"/>
     </row>
     <row r="29" spans="1:62" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A29" s="18" t="s">
+      <c r="A29" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="B29" s="18"/>
-      <c r="C29" s="18"/>
-      <c r="D29" s="12">
+      <c r="B29" s="22"/>
+      <c r="C29" s="22"/>
+      <c r="D29" s="17">
         <v>6</v>
       </c>
-      <c r="E29" s="12"/>
-      <c r="F29" s="13"/>
+      <c r="E29" s="17"/>
+      <c r="F29" s="18"/>
       <c r="G29" s="10">
-        <v>45756</v>
+        <v>45777</v>
       </c>
       <c r="AH29" s="7"/>
       <c r="AI29" s="7"/>
@@ -1445,14 +1451,14 @@
       <c r="BD29" s="3"/>
     </row>
     <row r="30" spans="1:62" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A30" s="18"/>
-      <c r="B30" s="18"/>
-      <c r="C30" s="18"/>
-      <c r="D30" s="14"/>
-      <c r="E30" s="14"/>
-      <c r="F30" s="15"/>
+      <c r="A30" s="22"/>
+      <c r="B30" s="22"/>
+      <c r="C30" s="22"/>
+      <c r="D30" s="19"/>
+      <c r="E30" s="19"/>
+      <c r="F30" s="20"/>
       <c r="G30" s="10">
-        <v>45763</v>
+        <v>45778</v>
       </c>
       <c r="AN30" s="7"/>
       <c r="AO30" s="7"/>
@@ -1465,16 +1471,16 @@
       <c r="BD30" s="3"/>
     </row>
     <row r="31" spans="1:62" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A31" s="18" t="s">
+      <c r="A31" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="B31" s="18"/>
-      <c r="C31" s="18"/>
-      <c r="D31" s="12">
+      <c r="B31" s="22"/>
+      <c r="C31" s="22"/>
+      <c r="D31" s="17">
         <v>6</v>
       </c>
-      <c r="E31" s="12"/>
-      <c r="F31" s="13"/>
+      <c r="E31" s="17"/>
+      <c r="F31" s="18"/>
       <c r="G31" s="10">
         <v>45777</v>
       </c>
@@ -1490,12 +1496,12 @@
       <c r="BJ31" s="3"/>
     </row>
     <row r="32" spans="1:62" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A32" s="18"/>
-      <c r="B32" s="18"/>
-      <c r="C32" s="18"/>
-      <c r="D32" s="14"/>
-      <c r="E32" s="14"/>
-      <c r="F32" s="15"/>
+      <c r="A32" s="22"/>
+      <c r="B32" s="22"/>
+      <c r="C32" s="22"/>
+      <c r="D32" s="19"/>
+      <c r="E32" s="19"/>
+      <c r="F32" s="20"/>
       <c r="G32" s="10">
         <v>45778</v>
       </c>
@@ -1511,16 +1517,16 @@
       <c r="BJ32" s="3"/>
     </row>
     <row r="33" spans="1:73" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A33" s="17" t="s">
+      <c r="A33" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="17"/>
-      <c r="C33" s="17"/>
-      <c r="D33" s="12">
+      <c r="B33" s="23"/>
+      <c r="C33" s="23"/>
+      <c r="D33" s="17">
         <v>2</v>
       </c>
-      <c r="E33" s="12"/>
-      <c r="F33" s="13"/>
+      <c r="E33" s="17"/>
+      <c r="F33" s="18"/>
       <c r="G33" s="10">
         <v>45785</v>
       </c>
@@ -1528,12 +1534,12 @@
       <c r="BL33" s="4"/>
     </row>
     <row r="34" spans="1:73" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A34" s="17"/>
-      <c r="B34" s="17"/>
-      <c r="C34" s="17"/>
-      <c r="D34" s="14"/>
-      <c r="E34" s="14"/>
-      <c r="F34" s="15"/>
+      <c r="A34" s="23"/>
+      <c r="B34" s="23"/>
+      <c r="C34" s="23"/>
+      <c r="D34" s="19"/>
+      <c r="E34" s="19"/>
+      <c r="F34" s="20"/>
       <c r="G34" s="10">
         <v>45785</v>
       </c>
@@ -1541,16 +1547,16 @@
       <c r="BL34" s="4"/>
     </row>
     <row r="35" spans="1:73" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A35" s="17" t="s">
+      <c r="A35" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="B35" s="17"/>
-      <c r="C35" s="17"/>
-      <c r="D35" s="12">
+      <c r="B35" s="23"/>
+      <c r="C35" s="23"/>
+      <c r="D35" s="17">
         <v>2</v>
       </c>
-      <c r="E35" s="12"/>
-      <c r="F35" s="13"/>
+      <c r="E35" s="17"/>
+      <c r="F35" s="18"/>
       <c r="G35" s="10">
         <v>45785</v>
       </c>
@@ -1558,12 +1564,12 @@
       <c r="BL35" s="4"/>
     </row>
     <row r="36" spans="1:73" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A36" s="17"/>
-      <c r="B36" s="17"/>
-      <c r="C36" s="17"/>
-      <c r="D36" s="14"/>
-      <c r="E36" s="14"/>
-      <c r="F36" s="15"/>
+      <c r="A36" s="23"/>
+      <c r="B36" s="23"/>
+      <c r="C36" s="23"/>
+      <c r="D36" s="19"/>
+      <c r="E36" s="19"/>
+      <c r="F36" s="20"/>
       <c r="G36" s="10">
         <v>45785</v>
       </c>
@@ -1571,16 +1577,16 @@
       <c r="BL36" s="4"/>
     </row>
     <row r="37" spans="1:73" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A37" s="17" t="s">
+      <c r="A37" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="B37" s="17"/>
-      <c r="C37" s="17"/>
-      <c r="D37" s="12">
+      <c r="B37" s="23"/>
+      <c r="C37" s="23"/>
+      <c r="D37" s="17">
         <v>2</v>
       </c>
-      <c r="E37" s="12"/>
-      <c r="F37" s="13"/>
+      <c r="E37" s="17"/>
+      <c r="F37" s="18"/>
       <c r="G37" s="10">
         <v>45785</v>
       </c>
@@ -1588,12 +1594,12 @@
       <c r="BL37" s="4"/>
     </row>
     <row r="38" spans="1:73" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A38" s="17"/>
-      <c r="B38" s="17"/>
-      <c r="C38" s="17"/>
-      <c r="D38" s="14"/>
-      <c r="E38" s="14"/>
-      <c r="F38" s="15"/>
+      <c r="A38" s="23"/>
+      <c r="B38" s="23"/>
+      <c r="C38" s="23"/>
+      <c r="D38" s="19"/>
+      <c r="E38" s="19"/>
+      <c r="F38" s="20"/>
       <c r="G38" s="10">
         <v>45785</v>
       </c>
@@ -1601,16 +1607,16 @@
       <c r="BL38" s="4"/>
     </row>
     <row r="39" spans="1:73" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A39" s="17" t="s">
+      <c r="A39" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="B39" s="17"/>
-      <c r="C39" s="17"/>
-      <c r="D39" s="12">
+      <c r="B39" s="23"/>
+      <c r="C39" s="23"/>
+      <c r="D39" s="17">
         <v>2</v>
       </c>
-      <c r="E39" s="12"/>
-      <c r="F39" s="13"/>
+      <c r="E39" s="17"/>
+      <c r="F39" s="18"/>
       <c r="G39" s="10">
         <v>45785</v>
       </c>
@@ -1618,12 +1624,12 @@
       <c r="BL39" s="4"/>
     </row>
     <row r="40" spans="1:73" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A40" s="17"/>
-      <c r="B40" s="17"/>
-      <c r="C40" s="17"/>
-      <c r="D40" s="14"/>
-      <c r="E40" s="14"/>
-      <c r="F40" s="15"/>
+      <c r="A40" s="23"/>
+      <c r="B40" s="23"/>
+      <c r="C40" s="23"/>
+      <c r="D40" s="19"/>
+      <c r="E40" s="19"/>
+      <c r="F40" s="20"/>
       <c r="G40" s="10">
         <v>45785</v>
       </c>
@@ -1631,16 +1637,16 @@
       <c r="BL40" s="4"/>
     </row>
     <row r="41" spans="1:73" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A41" s="11" t="s">
+      <c r="A41" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="B41" s="11"/>
-      <c r="C41" s="11"/>
-      <c r="D41" s="12">
+      <c r="B41" s="24"/>
+      <c r="C41" s="24"/>
+      <c r="D41" s="17">
         <v>4</v>
       </c>
-      <c r="E41" s="12"/>
-      <c r="F41" s="13"/>
+      <c r="E41" s="17"/>
+      <c r="F41" s="18"/>
       <c r="G41" s="10">
         <v>45792</v>
       </c>
@@ -1650,14 +1656,14 @@
       <c r="BP41" s="5"/>
     </row>
     <row r="42" spans="1:73" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A42" s="11"/>
-      <c r="B42" s="11"/>
-      <c r="C42" s="11"/>
-      <c r="D42" s="14"/>
-      <c r="E42" s="14"/>
-      <c r="F42" s="15"/>
+      <c r="A42" s="24"/>
+      <c r="B42" s="24"/>
+      <c r="C42" s="24"/>
+      <c r="D42" s="19"/>
+      <c r="E42" s="19"/>
+      <c r="F42" s="20"/>
       <c r="G42" s="10">
-        <v>45792</v>
+        <v>45799</v>
       </c>
       <c r="BM42" s="5"/>
       <c r="BN42" s="5"/>
@@ -1665,28 +1671,28 @@
       <c r="BP42" s="5"/>
     </row>
     <row r="43" spans="1:73" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A43" s="16" t="s">
+      <c r="A43" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="B43" s="16"/>
-      <c r="C43" s="16"/>
-      <c r="D43" s="12">
+      <c r="B43" s="25"/>
+      <c r="C43" s="25"/>
+      <c r="D43" s="17">
         <f>SUM(D3:F42)</f>
-        <v>74</v>
-      </c>
-      <c r="E43" s="12"/>
-      <c r="F43" s="13"/>
+        <v>78</v>
+      </c>
+      <c r="E43" s="17"/>
+      <c r="F43" s="18"/>
       <c r="G43" s="9">
         <v>45665</v>
       </c>
     </row>
     <row r="44" spans="1:73" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A44" s="16"/>
-      <c r="B44" s="16"/>
-      <c r="C44" s="16"/>
-      <c r="D44" s="14"/>
-      <c r="E44" s="14"/>
-      <c r="F44" s="15"/>
+      <c r="A44" s="25"/>
+      <c r="B44" s="25"/>
+      <c r="C44" s="25"/>
+      <c r="D44" s="19"/>
+      <c r="E44" s="19"/>
+      <c r="F44" s="20"/>
       <c r="G44" s="10">
         <v>45820</v>
       </c>
@@ -1758,17 +1764,17 @@
       <c r="BU44" s="7"/>
     </row>
     <row r="45" spans="1:73" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A45" s="16" t="s">
+      <c r="A45" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="B45" s="16"/>
-      <c r="C45" s="16"/>
-      <c r="D45" s="12">
+      <c r="B45" s="25"/>
+      <c r="C45" s="25"/>
+      <c r="D45" s="17">
         <f>SUM(D3:F42)</f>
-        <v>74</v>
-      </c>
-      <c r="E45" s="12"/>
-      <c r="F45" s="13"/>
+        <v>78</v>
+      </c>
+      <c r="E45" s="17"/>
+      <c r="F45" s="18"/>
       <c r="G45" s="9">
         <v>45665</v>
       </c>
@@ -1840,12 +1846,12 @@
       <c r="BU45" s="7"/>
     </row>
     <row r="46" spans="1:73" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A46" s="16"/>
-      <c r="B46" s="16"/>
-      <c r="C46" s="16"/>
-      <c r="D46" s="14"/>
-      <c r="E46" s="14"/>
-      <c r="F46" s="15"/>
+      <c r="A46" s="25"/>
+      <c r="B46" s="25"/>
+      <c r="C46" s="25"/>
+      <c r="D46" s="19"/>
+      <c r="E46" s="19"/>
+      <c r="F46" s="20"/>
       <c r="G46" s="10">
         <v>45820</v>
       </c>
@@ -1918,54 +1924,54 @@
     </row>
   </sheetData>
   <mergeCells count="48">
+    <mergeCell ref="A41:C42"/>
+    <mergeCell ref="D41:F42"/>
+    <mergeCell ref="A43:C44"/>
+    <mergeCell ref="D43:F44"/>
+    <mergeCell ref="A45:C46"/>
+    <mergeCell ref="D45:F46"/>
+    <mergeCell ref="A35:C36"/>
+    <mergeCell ref="D35:F36"/>
+    <mergeCell ref="A37:C38"/>
+    <mergeCell ref="D37:F38"/>
+    <mergeCell ref="A39:C40"/>
+    <mergeCell ref="D39:F40"/>
+    <mergeCell ref="A29:C30"/>
+    <mergeCell ref="D29:F30"/>
+    <mergeCell ref="A31:C32"/>
+    <mergeCell ref="D31:F32"/>
+    <mergeCell ref="A33:C34"/>
+    <mergeCell ref="D33:F34"/>
+    <mergeCell ref="A23:C24"/>
+    <mergeCell ref="D23:F24"/>
+    <mergeCell ref="A25:C26"/>
+    <mergeCell ref="D25:F26"/>
+    <mergeCell ref="A27:C28"/>
+    <mergeCell ref="D27:F28"/>
+    <mergeCell ref="A17:C18"/>
+    <mergeCell ref="D17:F18"/>
+    <mergeCell ref="A19:C20"/>
+    <mergeCell ref="D19:F20"/>
+    <mergeCell ref="A21:C22"/>
+    <mergeCell ref="D21:F22"/>
+    <mergeCell ref="A11:C12"/>
+    <mergeCell ref="D11:F12"/>
+    <mergeCell ref="A13:C14"/>
+    <mergeCell ref="D13:F14"/>
+    <mergeCell ref="A15:C16"/>
+    <mergeCell ref="D15:F16"/>
+    <mergeCell ref="A5:C6"/>
+    <mergeCell ref="D5:F6"/>
+    <mergeCell ref="A7:C8"/>
+    <mergeCell ref="D7:F8"/>
+    <mergeCell ref="A9:C10"/>
+    <mergeCell ref="D9:F10"/>
     <mergeCell ref="BD1:CZ2"/>
     <mergeCell ref="A1:C2"/>
     <mergeCell ref="D1:F2"/>
     <mergeCell ref="G1:BC2"/>
     <mergeCell ref="A3:C4"/>
     <mergeCell ref="D3:F4"/>
-    <mergeCell ref="A5:C6"/>
-    <mergeCell ref="D5:F6"/>
-    <mergeCell ref="A7:C8"/>
-    <mergeCell ref="D7:F8"/>
-    <mergeCell ref="A9:C10"/>
-    <mergeCell ref="D9:F10"/>
-    <mergeCell ref="A11:C12"/>
-    <mergeCell ref="D11:F12"/>
-    <mergeCell ref="A13:C14"/>
-    <mergeCell ref="D13:F14"/>
-    <mergeCell ref="A15:C16"/>
-    <mergeCell ref="D15:F16"/>
-    <mergeCell ref="A17:C18"/>
-    <mergeCell ref="D17:F18"/>
-    <mergeCell ref="A19:C20"/>
-    <mergeCell ref="D19:F20"/>
-    <mergeCell ref="A21:C22"/>
-    <mergeCell ref="D21:F22"/>
-    <mergeCell ref="A23:C24"/>
-    <mergeCell ref="D23:F24"/>
-    <mergeCell ref="A25:C26"/>
-    <mergeCell ref="D25:F26"/>
-    <mergeCell ref="A27:C28"/>
-    <mergeCell ref="D27:F28"/>
-    <mergeCell ref="A29:C30"/>
-    <mergeCell ref="D29:F30"/>
-    <mergeCell ref="A31:C32"/>
-    <mergeCell ref="D31:F32"/>
-    <mergeCell ref="A33:C34"/>
-    <mergeCell ref="D33:F34"/>
-    <mergeCell ref="A35:C36"/>
-    <mergeCell ref="D35:F36"/>
-    <mergeCell ref="A37:C38"/>
-    <mergeCell ref="D37:F38"/>
-    <mergeCell ref="A39:C40"/>
-    <mergeCell ref="D39:F40"/>
-    <mergeCell ref="A41:C42"/>
-    <mergeCell ref="D41:F42"/>
-    <mergeCell ref="A43:C44"/>
-    <mergeCell ref="D43:F44"/>
-    <mergeCell ref="A45:C46"/>
-    <mergeCell ref="D45:F46"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Sprint 4 documentazione + errori con desc
</commit_message>
<xml_diff>
--- a/7_Allegati/Gantt/Gantt_cons.xlsx
+++ b/7_Allegati/Gantt/Gantt_cons.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\M306\Progetto_CasaNote\7_Allegati\Gantt\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\M306\CasaNote\7_Allegati\Gantt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A92884E-66C0-4230-99CA-1079F0E7A2DC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{663241FF-37F8-449D-BFBB-D693CF4BDCD2}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="14025" xr2:uid="{285B56FD-1A67-4790-99DC-B99A42CD0DBC}"/>
   </bookViews>
@@ -359,8 +359,23 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -374,35 +389,20 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -731,232 +731,232 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:104" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24" t="s">
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
-      <c r="K1" s="23"/>
-      <c r="L1" s="23"/>
-      <c r="M1" s="23"/>
-      <c r="N1" s="23"/>
-      <c r="O1" s="23"/>
-      <c r="P1" s="23"/>
-      <c r="Q1" s="23"/>
-      <c r="R1" s="23"/>
-      <c r="S1" s="23"/>
-      <c r="T1" s="23"/>
-      <c r="U1" s="23"/>
-      <c r="V1" s="23"/>
-      <c r="W1" s="23"/>
-      <c r="X1" s="23"/>
-      <c r="Y1" s="23"/>
-      <c r="Z1" s="23"/>
-      <c r="AA1" s="23"/>
-      <c r="AB1" s="23"/>
-      <c r="AC1" s="23"/>
-      <c r="AD1" s="23"/>
-      <c r="AE1" s="23"/>
-      <c r="AF1" s="23"/>
-      <c r="AG1" s="23"/>
-      <c r="AH1" s="23"/>
-      <c r="AI1" s="23"/>
-      <c r="AJ1" s="23"/>
-      <c r="AK1" s="23"/>
-      <c r="AL1" s="23"/>
-      <c r="AM1" s="23"/>
-      <c r="AN1" s="23"/>
-      <c r="AO1" s="23"/>
-      <c r="AP1" s="23"/>
-      <c r="AQ1" s="23"/>
-      <c r="AR1" s="23"/>
-      <c r="AS1" s="23"/>
-      <c r="AT1" s="23"/>
-      <c r="AU1" s="23"/>
-      <c r="AV1" s="23"/>
-      <c r="AW1" s="23"/>
-      <c r="AX1" s="23"/>
-      <c r="AY1" s="23"/>
-      <c r="AZ1" s="23"/>
-      <c r="BA1" s="23"/>
-      <c r="BB1" s="23"/>
-      <c r="BC1" s="23"/>
-      <c r="BD1" s="23"/>
-      <c r="BE1" s="23"/>
-      <c r="BF1" s="23"/>
-      <c r="BG1" s="23"/>
-      <c r="BH1" s="23"/>
-      <c r="BI1" s="23"/>
-      <c r="BJ1" s="23"/>
-      <c r="BK1" s="23"/>
-      <c r="BL1" s="23"/>
-      <c r="BM1" s="23"/>
-      <c r="BN1" s="23"/>
-      <c r="BO1" s="23"/>
-      <c r="BP1" s="23"/>
-      <c r="BQ1" s="23"/>
-      <c r="BR1" s="23"/>
-      <c r="BS1" s="23"/>
-      <c r="BT1" s="23"/>
-      <c r="BU1" s="23"/>
-      <c r="BV1" s="23"/>
-      <c r="BW1" s="23"/>
-      <c r="BX1" s="23"/>
-      <c r="BY1" s="23"/>
-      <c r="BZ1" s="23"/>
-      <c r="CA1" s="23"/>
-      <c r="CB1" s="23"/>
-      <c r="CC1" s="23"/>
-      <c r="CD1" s="23"/>
-      <c r="CE1" s="23"/>
-      <c r="CF1" s="23"/>
-      <c r="CG1" s="23"/>
-      <c r="CH1" s="23"/>
-      <c r="CI1" s="23"/>
-      <c r="CJ1" s="23"/>
-      <c r="CK1" s="23"/>
-      <c r="CL1" s="23"/>
-      <c r="CM1" s="23"/>
-      <c r="CN1" s="23"/>
-      <c r="CO1" s="23"/>
-      <c r="CP1" s="23"/>
-      <c r="CQ1" s="23"/>
-      <c r="CR1" s="23"/>
-      <c r="CS1" s="23"/>
-      <c r="CT1" s="23"/>
-      <c r="CU1" s="23"/>
-      <c r="CV1" s="23"/>
-      <c r="CW1" s="23"/>
-      <c r="CX1" s="23"/>
-      <c r="CY1" s="23"/>
-      <c r="CZ1" s="23"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
+      <c r="J1" s="11"/>
+      <c r="K1" s="11"/>
+      <c r="L1" s="11"/>
+      <c r="M1" s="11"/>
+      <c r="N1" s="11"/>
+      <c r="O1" s="11"/>
+      <c r="P1" s="11"/>
+      <c r="Q1" s="11"/>
+      <c r="R1" s="11"/>
+      <c r="S1" s="11"/>
+      <c r="T1" s="11"/>
+      <c r="U1" s="11"/>
+      <c r="V1" s="11"/>
+      <c r="W1" s="11"/>
+      <c r="X1" s="11"/>
+      <c r="Y1" s="11"/>
+      <c r="Z1" s="11"/>
+      <c r="AA1" s="11"/>
+      <c r="AB1" s="11"/>
+      <c r="AC1" s="11"/>
+      <c r="AD1" s="11"/>
+      <c r="AE1" s="11"/>
+      <c r="AF1" s="11"/>
+      <c r="AG1" s="11"/>
+      <c r="AH1" s="11"/>
+      <c r="AI1" s="11"/>
+      <c r="AJ1" s="11"/>
+      <c r="AK1" s="11"/>
+      <c r="AL1" s="11"/>
+      <c r="AM1" s="11"/>
+      <c r="AN1" s="11"/>
+      <c r="AO1" s="11"/>
+      <c r="AP1" s="11"/>
+      <c r="AQ1" s="11"/>
+      <c r="AR1" s="11"/>
+      <c r="AS1" s="11"/>
+      <c r="AT1" s="11"/>
+      <c r="AU1" s="11"/>
+      <c r="AV1" s="11"/>
+      <c r="AW1" s="11"/>
+      <c r="AX1" s="11"/>
+      <c r="AY1" s="11"/>
+      <c r="AZ1" s="11"/>
+      <c r="BA1" s="11"/>
+      <c r="BB1" s="11"/>
+      <c r="BC1" s="11"/>
+      <c r="BD1" s="11"/>
+      <c r="BE1" s="11"/>
+      <c r="BF1" s="11"/>
+      <c r="BG1" s="11"/>
+      <c r="BH1" s="11"/>
+      <c r="BI1" s="11"/>
+      <c r="BJ1" s="11"/>
+      <c r="BK1" s="11"/>
+      <c r="BL1" s="11"/>
+      <c r="BM1" s="11"/>
+      <c r="BN1" s="11"/>
+      <c r="BO1" s="11"/>
+      <c r="BP1" s="11"/>
+      <c r="BQ1" s="11"/>
+      <c r="BR1" s="11"/>
+      <c r="BS1" s="11"/>
+      <c r="BT1" s="11"/>
+      <c r="BU1" s="11"/>
+      <c r="BV1" s="11"/>
+      <c r="BW1" s="11"/>
+      <c r="BX1" s="11"/>
+      <c r="BY1" s="11"/>
+      <c r="BZ1" s="11"/>
+      <c r="CA1" s="11"/>
+      <c r="CB1" s="11"/>
+      <c r="CC1" s="11"/>
+      <c r="CD1" s="11"/>
+      <c r="CE1" s="11"/>
+      <c r="CF1" s="11"/>
+      <c r="CG1" s="11"/>
+      <c r="CH1" s="11"/>
+      <c r="CI1" s="11"/>
+      <c r="CJ1" s="11"/>
+      <c r="CK1" s="11"/>
+      <c r="CL1" s="11"/>
+      <c r="CM1" s="11"/>
+      <c r="CN1" s="11"/>
+      <c r="CO1" s="11"/>
+      <c r="CP1" s="11"/>
+      <c r="CQ1" s="11"/>
+      <c r="CR1" s="11"/>
+      <c r="CS1" s="11"/>
+      <c r="CT1" s="11"/>
+      <c r="CU1" s="11"/>
+      <c r="CV1" s="11"/>
+      <c r="CW1" s="11"/>
+      <c r="CX1" s="11"/>
+      <c r="CY1" s="11"/>
+      <c r="CZ1" s="11"/>
     </row>
     <row r="2" spans="1:104" ht="16.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="25"/>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
-      <c r="I2" s="23"/>
-      <c r="J2" s="23"/>
-      <c r="K2" s="23"/>
-      <c r="L2" s="23"/>
-      <c r="M2" s="23"/>
-      <c r="N2" s="23"/>
-      <c r="O2" s="23"/>
-      <c r="P2" s="23"/>
-      <c r="Q2" s="23"/>
-      <c r="R2" s="23"/>
-      <c r="S2" s="23"/>
-      <c r="T2" s="23"/>
-      <c r="U2" s="23"/>
-      <c r="V2" s="23"/>
-      <c r="W2" s="23"/>
-      <c r="X2" s="23"/>
-      <c r="Y2" s="23"/>
-      <c r="Z2" s="23"/>
-      <c r="AA2" s="23"/>
-      <c r="AB2" s="23"/>
-      <c r="AC2" s="23"/>
-      <c r="AD2" s="23"/>
-      <c r="AE2" s="23"/>
-      <c r="AF2" s="23"/>
-      <c r="AG2" s="23"/>
-      <c r="AH2" s="23"/>
-      <c r="AI2" s="23"/>
-      <c r="AJ2" s="23"/>
-      <c r="AK2" s="23"/>
-      <c r="AL2" s="23"/>
-      <c r="AM2" s="23"/>
-      <c r="AN2" s="23"/>
-      <c r="AO2" s="23"/>
-      <c r="AP2" s="23"/>
-      <c r="AQ2" s="23"/>
-      <c r="AR2" s="23"/>
-      <c r="AS2" s="23"/>
-      <c r="AT2" s="23"/>
-      <c r="AU2" s="23"/>
-      <c r="AV2" s="23"/>
-      <c r="AW2" s="23"/>
-      <c r="AX2" s="23"/>
-      <c r="AY2" s="23"/>
-      <c r="AZ2" s="23"/>
-      <c r="BA2" s="23"/>
-      <c r="BB2" s="23"/>
-      <c r="BC2" s="23"/>
-      <c r="BD2" s="23"/>
-      <c r="BE2" s="23"/>
-      <c r="BF2" s="23"/>
-      <c r="BG2" s="23"/>
-      <c r="BH2" s="23"/>
-      <c r="BI2" s="23"/>
-      <c r="BJ2" s="23"/>
-      <c r="BK2" s="23"/>
-      <c r="BL2" s="23"/>
-      <c r="BM2" s="23"/>
-      <c r="BN2" s="23"/>
-      <c r="BO2" s="23"/>
-      <c r="BP2" s="23"/>
-      <c r="BQ2" s="23"/>
-      <c r="BR2" s="23"/>
-      <c r="BS2" s="23"/>
-      <c r="BT2" s="23"/>
-      <c r="BU2" s="23"/>
-      <c r="BV2" s="23"/>
-      <c r="BW2" s="23"/>
-      <c r="BX2" s="23"/>
-      <c r="BY2" s="23"/>
-      <c r="BZ2" s="23"/>
-      <c r="CA2" s="23"/>
-      <c r="CB2" s="23"/>
-      <c r="CC2" s="23"/>
-      <c r="CD2" s="23"/>
-      <c r="CE2" s="23"/>
-      <c r="CF2" s="23"/>
-      <c r="CG2" s="23"/>
-      <c r="CH2" s="23"/>
-      <c r="CI2" s="23"/>
-      <c r="CJ2" s="23"/>
-      <c r="CK2" s="23"/>
-      <c r="CL2" s="23"/>
-      <c r="CM2" s="23"/>
-      <c r="CN2" s="23"/>
-      <c r="CO2" s="23"/>
-      <c r="CP2" s="23"/>
-      <c r="CQ2" s="23"/>
-      <c r="CR2" s="23"/>
-      <c r="CS2" s="23"/>
-      <c r="CT2" s="23"/>
-      <c r="CU2" s="23"/>
-      <c r="CV2" s="23"/>
-      <c r="CW2" s="23"/>
-      <c r="CX2" s="23"/>
-      <c r="CY2" s="23"/>
-      <c r="CZ2" s="23"/>
+      <c r="A2" s="13"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="11"/>
+      <c r="H2" s="11"/>
+      <c r="I2" s="11"/>
+      <c r="J2" s="11"/>
+      <c r="K2" s="11"/>
+      <c r="L2" s="11"/>
+      <c r="M2" s="11"/>
+      <c r="N2" s="11"/>
+      <c r="O2" s="11"/>
+      <c r="P2" s="11"/>
+      <c r="Q2" s="11"/>
+      <c r="R2" s="11"/>
+      <c r="S2" s="11"/>
+      <c r="T2" s="11"/>
+      <c r="U2" s="11"/>
+      <c r="V2" s="11"/>
+      <c r="W2" s="11"/>
+      <c r="X2" s="11"/>
+      <c r="Y2" s="11"/>
+      <c r="Z2" s="11"/>
+      <c r="AA2" s="11"/>
+      <c r="AB2" s="11"/>
+      <c r="AC2" s="11"/>
+      <c r="AD2" s="11"/>
+      <c r="AE2" s="11"/>
+      <c r="AF2" s="11"/>
+      <c r="AG2" s="11"/>
+      <c r="AH2" s="11"/>
+      <c r="AI2" s="11"/>
+      <c r="AJ2" s="11"/>
+      <c r="AK2" s="11"/>
+      <c r="AL2" s="11"/>
+      <c r="AM2" s="11"/>
+      <c r="AN2" s="11"/>
+      <c r="AO2" s="11"/>
+      <c r="AP2" s="11"/>
+      <c r="AQ2" s="11"/>
+      <c r="AR2" s="11"/>
+      <c r="AS2" s="11"/>
+      <c r="AT2" s="11"/>
+      <c r="AU2" s="11"/>
+      <c r="AV2" s="11"/>
+      <c r="AW2" s="11"/>
+      <c r="AX2" s="11"/>
+      <c r="AY2" s="11"/>
+      <c r="AZ2" s="11"/>
+      <c r="BA2" s="11"/>
+      <c r="BB2" s="11"/>
+      <c r="BC2" s="11"/>
+      <c r="BD2" s="11"/>
+      <c r="BE2" s="11"/>
+      <c r="BF2" s="11"/>
+      <c r="BG2" s="11"/>
+      <c r="BH2" s="11"/>
+      <c r="BI2" s="11"/>
+      <c r="BJ2" s="11"/>
+      <c r="BK2" s="11"/>
+      <c r="BL2" s="11"/>
+      <c r="BM2" s="11"/>
+      <c r="BN2" s="11"/>
+      <c r="BO2" s="11"/>
+      <c r="BP2" s="11"/>
+      <c r="BQ2" s="11"/>
+      <c r="BR2" s="11"/>
+      <c r="BS2" s="11"/>
+      <c r="BT2" s="11"/>
+      <c r="BU2" s="11"/>
+      <c r="BV2" s="11"/>
+      <c r="BW2" s="11"/>
+      <c r="BX2" s="11"/>
+      <c r="BY2" s="11"/>
+      <c r="BZ2" s="11"/>
+      <c r="CA2" s="11"/>
+      <c r="CB2" s="11"/>
+      <c r="CC2" s="11"/>
+      <c r="CD2" s="11"/>
+      <c r="CE2" s="11"/>
+      <c r="CF2" s="11"/>
+      <c r="CG2" s="11"/>
+      <c r="CH2" s="11"/>
+      <c r="CI2" s="11"/>
+      <c r="CJ2" s="11"/>
+      <c r="CK2" s="11"/>
+      <c r="CL2" s="11"/>
+      <c r="CM2" s="11"/>
+      <c r="CN2" s="11"/>
+      <c r="CO2" s="11"/>
+      <c r="CP2" s="11"/>
+      <c r="CQ2" s="11"/>
+      <c r="CR2" s="11"/>
+      <c r="CS2" s="11"/>
+      <c r="CT2" s="11"/>
+      <c r="CU2" s="11"/>
+      <c r="CV2" s="11"/>
+      <c r="CW2" s="11"/>
+      <c r="CX2" s="11"/>
+      <c r="CY2" s="11"/>
+      <c r="CZ2" s="11"/>
     </row>
     <row r="3" spans="1:104" ht="29.25" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="21">
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="15">
         <v>3</v>
       </c>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="16"/>
       <c r="G3" s="8">
         <v>45665</v>
       </c>
@@ -965,12 +965,12 @@
       <c r="J3" s="1"/>
     </row>
     <row r="4" spans="1:104" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A4" s="20"/>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
+      <c r="A4" s="14"/>
+      <c r="B4" s="14"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="16"/>
       <c r="G4" s="9">
         <v>45665</v>
       </c>
@@ -979,16 +979,16 @@
       <c r="J4" s="1"/>
     </row>
     <row r="5" spans="1:104" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="20" t="s">
+      <c r="A5" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="20"/>
-      <c r="C5" s="20"/>
-      <c r="D5" s="21">
+      <c r="B5" s="14"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="15">
         <v>3</v>
       </c>
-      <c r="E5" s="22"/>
-      <c r="F5" s="22"/>
+      <c r="E5" s="16"/>
+      <c r="F5" s="16"/>
       <c r="G5" s="9">
         <v>45665</v>
       </c>
@@ -997,12 +997,12 @@
       <c r="M5" s="1"/>
     </row>
     <row r="6" spans="1:104" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A6" s="20"/>
-      <c r="B6" s="20"/>
-      <c r="C6" s="20"/>
-      <c r="D6" s="21"/>
-      <c r="E6" s="22"/>
-      <c r="F6" s="22"/>
+      <c r="A6" s="14"/>
+      <c r="B6" s="14"/>
+      <c r="C6" s="14"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="16"/>
       <c r="G6" s="9">
         <v>45665</v>
       </c>
@@ -1011,16 +1011,16 @@
       <c r="M6" s="1"/>
     </row>
     <row r="7" spans="1:104" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A7" s="20" t="s">
+      <c r="A7" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="20"/>
-      <c r="C7" s="20"/>
-      <c r="D7" s="12">
+      <c r="B7" s="14"/>
+      <c r="C7" s="14"/>
+      <c r="D7" s="17">
         <v>3</v>
       </c>
-      <c r="E7" s="12"/>
-      <c r="F7" s="13"/>
+      <c r="E7" s="17"/>
+      <c r="F7" s="18"/>
       <c r="G7" s="10">
         <v>45665</v>
       </c>
@@ -1029,12 +1029,12 @@
       <c r="P7" s="1"/>
     </row>
     <row r="8" spans="1:104" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A8" s="20"/>
-      <c r="B8" s="20"/>
-      <c r="C8" s="20"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="15"/>
+      <c r="A8" s="14"/>
+      <c r="B8" s="14"/>
+      <c r="C8" s="14"/>
+      <c r="D8" s="19"/>
+      <c r="E8" s="19"/>
+      <c r="F8" s="20"/>
       <c r="G8" s="10">
         <v>45672</v>
       </c>
@@ -1043,16 +1043,16 @@
       <c r="P8" s="1"/>
     </row>
     <row r="9" spans="1:104" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="19"/>
-      <c r="C9" s="19"/>
-      <c r="D9" s="12">
+      <c r="B9" s="21"/>
+      <c r="C9" s="21"/>
+      <c r="D9" s="17">
         <v>2</v>
       </c>
-      <c r="E9" s="12"/>
-      <c r="F9" s="13"/>
+      <c r="E9" s="17"/>
+      <c r="F9" s="18"/>
       <c r="G9" s="9">
         <v>45672</v>
       </c>
@@ -1061,12 +1061,12 @@
       <c r="S9" s="2"/>
     </row>
     <row r="10" spans="1:104" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A10" s="19"/>
-      <c r="B10" s="19"/>
-      <c r="C10" s="19"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="14"/>
-      <c r="F10" s="15"/>
+      <c r="A10" s="21"/>
+      <c r="B10" s="21"/>
+      <c r="C10" s="21"/>
+      <c r="D10" s="19"/>
+      <c r="E10" s="19"/>
+      <c r="F10" s="20"/>
       <c r="G10" s="9">
         <v>45679</v>
       </c>
@@ -1075,16 +1075,16 @@
       <c r="S10" s="2"/>
     </row>
     <row r="11" spans="1:104" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="B11" s="19"/>
-      <c r="C11" s="19"/>
-      <c r="D11" s="12">
+      <c r="B11" s="21"/>
+      <c r="C11" s="21"/>
+      <c r="D11" s="17">
         <v>2</v>
       </c>
-      <c r="E11" s="12"/>
-      <c r="F11" s="13"/>
+      <c r="E11" s="17"/>
+      <c r="F11" s="18"/>
       <c r="G11" s="9">
         <v>45672</v>
       </c>
@@ -1092,12 +1092,12 @@
       <c r="U11" s="2"/>
     </row>
     <row r="12" spans="1:104" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A12" s="19"/>
-      <c r="B12" s="19"/>
-      <c r="C12" s="19"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="15"/>
+      <c r="A12" s="21"/>
+      <c r="B12" s="21"/>
+      <c r="C12" s="21"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="20"/>
       <c r="G12" s="9">
         <v>45679</v>
       </c>
@@ -1105,16 +1105,16 @@
       <c r="U12" s="2"/>
     </row>
     <row r="13" spans="1:104" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A13" s="19" t="s">
+      <c r="A13" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="B13" s="19"/>
-      <c r="C13" s="19"/>
-      <c r="D13" s="12">
+      <c r="B13" s="21"/>
+      <c r="C13" s="21"/>
+      <c r="D13" s="17">
         <v>2</v>
       </c>
-      <c r="E13" s="12"/>
-      <c r="F13" s="13"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="18"/>
       <c r="G13" s="9">
         <v>45672</v>
       </c>
@@ -1122,12 +1122,12 @@
       <c r="W13" s="2"/>
     </row>
     <row r="14" spans="1:104" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A14" s="19"/>
-      <c r="B14" s="19"/>
-      <c r="C14" s="19"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="15"/>
+      <c r="A14" s="21"/>
+      <c r="B14" s="21"/>
+      <c r="C14" s="21"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="20"/>
       <c r="G14" s="9">
         <v>45679</v>
       </c>
@@ -1135,16 +1135,16 @@
       <c r="W14" s="2"/>
     </row>
     <row r="15" spans="1:104" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A15" s="19" t="s">
+      <c r="A15" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="B15" s="19"/>
-      <c r="C15" s="19"/>
-      <c r="D15" s="12">
+      <c r="B15" s="21"/>
+      <c r="C15" s="21"/>
+      <c r="D15" s="17">
         <v>2</v>
       </c>
-      <c r="E15" s="12"/>
-      <c r="F15" s="13"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="18"/>
       <c r="G15" s="9">
         <v>45679</v>
       </c>
@@ -1152,12 +1152,12 @@
       <c r="Y15" s="2"/>
     </row>
     <row r="16" spans="1:104" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A16" s="19"/>
-      <c r="B16" s="19"/>
-      <c r="C16" s="19"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14"/>
-      <c r="F16" s="15"/>
+      <c r="A16" s="21"/>
+      <c r="B16" s="21"/>
+      <c r="C16" s="21"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="20"/>
       <c r="G16" s="10">
         <v>45693</v>
       </c>
@@ -1165,16 +1165,16 @@
       <c r="Y16" s="2"/>
     </row>
     <row r="17" spans="1:65" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A17" s="19" t="s">
+      <c r="A17" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="B17" s="19"/>
-      <c r="C17" s="19"/>
-      <c r="D17" s="12">
+      <c r="B17" s="21"/>
+      <c r="C17" s="21"/>
+      <c r="D17" s="17">
         <v>2</v>
       </c>
-      <c r="E17" s="12"/>
-      <c r="F17" s="13"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="18"/>
       <c r="G17" s="10">
         <v>45693</v>
       </c>
@@ -1182,12 +1182,12 @@
       <c r="AA17" s="2"/>
     </row>
     <row r="18" spans="1:65" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A18" s="19"/>
-      <c r="B18" s="19"/>
-      <c r="C18" s="19"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="15"/>
+      <c r="A18" s="21"/>
+      <c r="B18" s="21"/>
+      <c r="C18" s="21"/>
+      <c r="D18" s="19"/>
+      <c r="E18" s="19"/>
+      <c r="F18" s="20"/>
       <c r="G18" s="10">
         <v>45693</v>
       </c>
@@ -1195,16 +1195,16 @@
       <c r="AA18" s="2"/>
     </row>
     <row r="19" spans="1:65" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A19" s="19" t="s">
+      <c r="A19" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="B19" s="19"/>
-      <c r="C19" s="19"/>
-      <c r="D19" s="12">
+      <c r="B19" s="21"/>
+      <c r="C19" s="21"/>
+      <c r="D19" s="17">
         <v>2</v>
       </c>
-      <c r="E19" s="12"/>
-      <c r="F19" s="13"/>
+      <c r="E19" s="17"/>
+      <c r="F19" s="18"/>
       <c r="G19" s="10">
         <v>45693</v>
       </c>
@@ -1212,12 +1212,12 @@
       <c r="AA19" s="2"/>
     </row>
     <row r="20" spans="1:65" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A20" s="19"/>
-      <c r="B20" s="19"/>
-      <c r="C20" s="19"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14"/>
-      <c r="F20" s="15"/>
+      <c r="A20" s="21"/>
+      <c r="B20" s="21"/>
+      <c r="C20" s="21"/>
+      <c r="D20" s="19"/>
+      <c r="E20" s="19"/>
+      <c r="F20" s="20"/>
       <c r="G20" s="10">
         <v>45693</v>
       </c>
@@ -1225,16 +1225,16 @@
       <c r="AA20" s="2"/>
     </row>
     <row r="21" spans="1:65" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A21" s="18" t="s">
+      <c r="A21" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="B21" s="18"/>
-      <c r="C21" s="18"/>
-      <c r="D21" s="12">
+      <c r="B21" s="22"/>
+      <c r="C21" s="22"/>
+      <c r="D21" s="17">
         <v>6</v>
       </c>
-      <c r="E21" s="12"/>
-      <c r="F21" s="13"/>
+      <c r="E21" s="17"/>
+      <c r="F21" s="18"/>
       <c r="G21" s="10">
         <v>45700</v>
       </c>
@@ -1246,12 +1246,12 @@
       <c r="AG21" s="3"/>
     </row>
     <row r="22" spans="1:65" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A22" s="18"/>
-      <c r="B22" s="18"/>
-      <c r="C22" s="18"/>
-      <c r="D22" s="14"/>
-      <c r="E22" s="14"/>
-      <c r="F22" s="15"/>
+      <c r="A22" s="22"/>
+      <c r="B22" s="22"/>
+      <c r="C22" s="22"/>
+      <c r="D22" s="19"/>
+      <c r="E22" s="19"/>
+      <c r="F22" s="20"/>
       <c r="G22" s="10">
         <v>45714</v>
       </c>
@@ -1263,16 +1263,16 @@
       <c r="AG22" s="3"/>
     </row>
     <row r="23" spans="1:65" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A23" s="18" t="s">
+      <c r="A23" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="B23" s="18"/>
-      <c r="C23" s="18"/>
-      <c r="D23" s="12">
+      <c r="B23" s="22"/>
+      <c r="C23" s="22"/>
+      <c r="D23" s="17">
         <v>5</v>
       </c>
-      <c r="E23" s="12"/>
-      <c r="F23" s="13"/>
+      <c r="E23" s="17"/>
+      <c r="F23" s="18"/>
       <c r="G23" s="10">
         <v>45700</v>
       </c>
@@ -1287,12 +1287,12 @@
       <c r="AM23" s="7"/>
     </row>
     <row r="24" spans="1:65" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A24" s="18"/>
-      <c r="B24" s="18"/>
-      <c r="C24" s="18"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="14"/>
-      <c r="F24" s="15"/>
+      <c r="A24" s="22"/>
+      <c r="B24" s="22"/>
+      <c r="C24" s="22"/>
+      <c r="D24" s="19"/>
+      <c r="E24" s="19"/>
+      <c r="F24" s="20"/>
       <c r="G24" s="10">
         <v>45714</v>
       </c>
@@ -1307,16 +1307,16 @@
       <c r="AM24" s="7"/>
     </row>
     <row r="25" spans="1:65" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A25" s="18" t="s">
+      <c r="A25" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="B25" s="18"/>
-      <c r="C25" s="18"/>
-      <c r="D25" s="12">
+      <c r="B25" s="22"/>
+      <c r="C25" s="22"/>
+      <c r="D25" s="17">
         <v>14</v>
       </c>
-      <c r="E25" s="12"/>
-      <c r="F25" s="13"/>
+      <c r="E25" s="17"/>
+      <c r="F25" s="18"/>
       <c r="G25" s="10">
         <v>45721</v>
       </c>
@@ -1340,12 +1340,12 @@
       <c r="BA25" s="3"/>
     </row>
     <row r="26" spans="1:65" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A26" s="18"/>
-      <c r="B26" s="18"/>
-      <c r="C26" s="18"/>
-      <c r="D26" s="14"/>
-      <c r="E26" s="14"/>
-      <c r="F26" s="15"/>
+      <c r="A26" s="22"/>
+      <c r="B26" s="22"/>
+      <c r="C26" s="22"/>
+      <c r="D26" s="19"/>
+      <c r="E26" s="19"/>
+      <c r="F26" s="20"/>
       <c r="G26" s="10">
         <v>45778</v>
       </c>
@@ -1369,16 +1369,16 @@
       <c r="BA26" s="3"/>
     </row>
     <row r="27" spans="1:65" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A27" s="18" t="s">
+      <c r="A27" s="22" t="s">
         <v>23</v>
       </c>
-      <c r="B27" s="18"/>
-      <c r="C27" s="18"/>
-      <c r="D27" s="12">
+      <c r="B27" s="22"/>
+      <c r="C27" s="22"/>
+      <c r="D27" s="17">
         <v>14</v>
       </c>
-      <c r="E27" s="12"/>
-      <c r="F27" s="13"/>
+      <c r="E27" s="17"/>
+      <c r="F27" s="18"/>
       <c r="G27" s="10">
         <v>45742</v>
       </c>
@@ -1403,16 +1403,20 @@
       <c r="BE27" s="3"/>
       <c r="BF27" s="3"/>
       <c r="BG27" s="3"/>
+      <c r="BH27" s="3"/>
+      <c r="BI27" s="3"/>
+      <c r="BJ27" s="3"/>
+      <c r="BK27" s="3"/>
     </row>
     <row r="28" spans="1:65" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A28" s="18"/>
-      <c r="B28" s="18"/>
-      <c r="C28" s="18"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="14"/>
-      <c r="F28" s="15"/>
+      <c r="A28" s="22"/>
+      <c r="B28" s="22"/>
+      <c r="C28" s="22"/>
+      <c r="D28" s="19"/>
+      <c r="E28" s="19"/>
+      <c r="F28" s="20"/>
       <c r="G28" s="10">
-        <v>45785</v>
+        <v>45798</v>
       </c>
       <c r="AH28" s="7"/>
       <c r="AI28" s="7"/>
@@ -1435,18 +1439,22 @@
       <c r="BE28" s="3"/>
       <c r="BF28" s="3"/>
       <c r="BG28" s="3"/>
+      <c r="BH28" s="3"/>
+      <c r="BI28" s="3"/>
+      <c r="BJ28" s="3"/>
+      <c r="BK28" s="3"/>
     </row>
     <row r="29" spans="1:65" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A29" s="18" t="s">
+      <c r="A29" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="B29" s="18"/>
-      <c r="C29" s="18"/>
-      <c r="D29" s="12">
+      <c r="B29" s="22"/>
+      <c r="C29" s="22"/>
+      <c r="D29" s="17">
         <v>6</v>
       </c>
-      <c r="E29" s="12"/>
-      <c r="F29" s="13"/>
+      <c r="E29" s="17"/>
+      <c r="F29" s="18"/>
       <c r="G29" s="10">
         <v>45777</v>
       </c>
@@ -1467,12 +1475,12 @@
       <c r="BM29" s="3"/>
     </row>
     <row r="30" spans="1:65" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A30" s="18"/>
-      <c r="B30" s="18"/>
-      <c r="C30" s="18"/>
-      <c r="D30" s="14"/>
-      <c r="E30" s="14"/>
-      <c r="F30" s="15"/>
+      <c r="A30" s="22"/>
+      <c r="B30" s="22"/>
+      <c r="C30" s="22"/>
+      <c r="D30" s="19"/>
+      <c r="E30" s="19"/>
+      <c r="F30" s="20"/>
       <c r="G30" s="10">
         <v>45778</v>
       </c>
@@ -1487,16 +1495,16 @@
       <c r="BM30" s="3"/>
     </row>
     <row r="31" spans="1:65" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A31" s="18" t="s">
+      <c r="A31" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="B31" s="18"/>
-      <c r="C31" s="18"/>
-      <c r="D31" s="12">
+      <c r="B31" s="22"/>
+      <c r="C31" s="22"/>
+      <c r="D31" s="17">
         <v>6</v>
       </c>
-      <c r="E31" s="12"/>
-      <c r="F31" s="13"/>
+      <c r="E31" s="17"/>
+      <c r="F31" s="18"/>
       <c r="G31" s="10">
         <v>45785</v>
       </c>
@@ -1512,12 +1520,12 @@
       <c r="BM31" s="3"/>
     </row>
     <row r="32" spans="1:65" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A32" s="18"/>
-      <c r="B32" s="18"/>
-      <c r="C32" s="18"/>
-      <c r="D32" s="14"/>
-      <c r="E32" s="14"/>
-      <c r="F32" s="15"/>
+      <c r="A32" s="22"/>
+      <c r="B32" s="22"/>
+      <c r="C32" s="22"/>
+      <c r="D32" s="19"/>
+      <c r="E32" s="19"/>
+      <c r="F32" s="20"/>
       <c r="G32" s="10">
         <v>45792</v>
       </c>
@@ -1533,16 +1541,16 @@
       <c r="BM32" s="3"/>
     </row>
     <row r="33" spans="1:73" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A33" s="17" t="s">
+      <c r="A33" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="17"/>
-      <c r="C33" s="17"/>
-      <c r="D33" s="12">
+      <c r="B33" s="23"/>
+      <c r="C33" s="23"/>
+      <c r="D33" s="17">
         <v>2</v>
       </c>
-      <c r="E33" s="12"/>
-      <c r="F33" s="13"/>
+      <c r="E33" s="17"/>
+      <c r="F33" s="18"/>
       <c r="G33" s="10">
         <v>45785</v>
       </c>
@@ -1550,12 +1558,12 @@
       <c r="BO33" s="4"/>
     </row>
     <row r="34" spans="1:73" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A34" s="17"/>
-      <c r="B34" s="17"/>
-      <c r="C34" s="17"/>
-      <c r="D34" s="14"/>
-      <c r="E34" s="14"/>
-      <c r="F34" s="15"/>
+      <c r="A34" s="23"/>
+      <c r="B34" s="23"/>
+      <c r="C34" s="23"/>
+      <c r="D34" s="19"/>
+      <c r="E34" s="19"/>
+      <c r="F34" s="20"/>
       <c r="G34" s="10">
         <v>45785</v>
       </c>
@@ -1563,16 +1571,16 @@
       <c r="BO34" s="4"/>
     </row>
     <row r="35" spans="1:73" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A35" s="17" t="s">
+      <c r="A35" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="B35" s="17"/>
-      <c r="C35" s="17"/>
-      <c r="D35" s="12">
+      <c r="B35" s="23"/>
+      <c r="C35" s="23"/>
+      <c r="D35" s="17">
         <v>2</v>
       </c>
-      <c r="E35" s="12"/>
-      <c r="F35" s="13"/>
+      <c r="E35" s="17"/>
+      <c r="F35" s="18"/>
       <c r="G35" s="10">
         <v>45785</v>
       </c>
@@ -1580,12 +1588,12 @@
       <c r="BO35" s="4"/>
     </row>
     <row r="36" spans="1:73" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A36" s="17"/>
-      <c r="B36" s="17"/>
-      <c r="C36" s="17"/>
-      <c r="D36" s="14"/>
-      <c r="E36" s="14"/>
-      <c r="F36" s="15"/>
+      <c r="A36" s="23"/>
+      <c r="B36" s="23"/>
+      <c r="C36" s="23"/>
+      <c r="D36" s="19"/>
+      <c r="E36" s="19"/>
+      <c r="F36" s="20"/>
       <c r="G36" s="10">
         <v>45785</v>
       </c>
@@ -1593,16 +1601,16 @@
       <c r="BO36" s="4"/>
     </row>
     <row r="37" spans="1:73" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A37" s="17" t="s">
+      <c r="A37" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="B37" s="17"/>
-      <c r="C37" s="17"/>
-      <c r="D37" s="12">
+      <c r="B37" s="23"/>
+      <c r="C37" s="23"/>
+      <c r="D37" s="17">
         <v>2</v>
       </c>
-      <c r="E37" s="12"/>
-      <c r="F37" s="13"/>
+      <c r="E37" s="17"/>
+      <c r="F37" s="18"/>
       <c r="G37" s="10">
         <v>45785</v>
       </c>
@@ -1610,12 +1618,12 @@
       <c r="BO37" s="4"/>
     </row>
     <row r="38" spans="1:73" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A38" s="17"/>
-      <c r="B38" s="17"/>
-      <c r="C38" s="17"/>
-      <c r="D38" s="14"/>
-      <c r="E38" s="14"/>
-      <c r="F38" s="15"/>
+      <c r="A38" s="23"/>
+      <c r="B38" s="23"/>
+      <c r="C38" s="23"/>
+      <c r="D38" s="19"/>
+      <c r="E38" s="19"/>
+      <c r="F38" s="20"/>
       <c r="G38" s="10">
         <v>45785</v>
       </c>
@@ -1623,16 +1631,16 @@
       <c r="BO38" s="4"/>
     </row>
     <row r="39" spans="1:73" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A39" s="17" t="s">
+      <c r="A39" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="B39" s="17"/>
-      <c r="C39" s="17"/>
-      <c r="D39" s="12">
+      <c r="B39" s="23"/>
+      <c r="C39" s="23"/>
+      <c r="D39" s="17">
         <v>2</v>
       </c>
-      <c r="E39" s="12"/>
-      <c r="F39" s="13"/>
+      <c r="E39" s="17"/>
+      <c r="F39" s="18"/>
       <c r="G39" s="10">
         <v>45785</v>
       </c>
@@ -1640,12 +1648,12 @@
       <c r="BO39" s="4"/>
     </row>
     <row r="40" spans="1:73" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A40" s="17"/>
-      <c r="B40" s="17"/>
-      <c r="C40" s="17"/>
-      <c r="D40" s="14"/>
-      <c r="E40" s="14"/>
-      <c r="F40" s="15"/>
+      <c r="A40" s="23"/>
+      <c r="B40" s="23"/>
+      <c r="C40" s="23"/>
+      <c r="D40" s="19"/>
+      <c r="E40" s="19"/>
+      <c r="F40" s="20"/>
       <c r="G40" s="10">
         <v>45785</v>
       </c>
@@ -1653,16 +1661,16 @@
       <c r="BO40" s="4"/>
     </row>
     <row r="41" spans="1:73" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A41" s="11" t="s">
+      <c r="A41" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="B41" s="11"/>
-      <c r="C41" s="11"/>
-      <c r="D41" s="12">
+      <c r="B41" s="24"/>
+      <c r="C41" s="24"/>
+      <c r="D41" s="17">
         <v>4</v>
       </c>
-      <c r="E41" s="12"/>
-      <c r="F41" s="13"/>
+      <c r="E41" s="17"/>
+      <c r="F41" s="18"/>
       <c r="G41" s="10">
         <v>45792</v>
       </c>
@@ -1672,12 +1680,12 @@
       <c r="BS41" s="5"/>
     </row>
     <row r="42" spans="1:73" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A42" s="11"/>
-      <c r="B42" s="11"/>
-      <c r="C42" s="11"/>
-      <c r="D42" s="14"/>
-      <c r="E42" s="14"/>
-      <c r="F42" s="15"/>
+      <c r="A42" s="24"/>
+      <c r="B42" s="24"/>
+      <c r="C42" s="24"/>
+      <c r="D42" s="19"/>
+      <c r="E42" s="19"/>
+      <c r="F42" s="20"/>
       <c r="G42" s="10">
         <v>45799</v>
       </c>
@@ -1687,28 +1695,28 @@
       <c r="BS42" s="5"/>
     </row>
     <row r="43" spans="1:73" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A43" s="16" t="s">
+      <c r="A43" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="B43" s="16"/>
-      <c r="C43" s="16"/>
-      <c r="D43" s="12">
+      <c r="B43" s="25"/>
+      <c r="C43" s="25"/>
+      <c r="D43" s="17">
         <f>SUM(D3:F42)</f>
         <v>84</v>
       </c>
-      <c r="E43" s="12"/>
-      <c r="F43" s="13"/>
+      <c r="E43" s="17"/>
+      <c r="F43" s="18"/>
       <c r="G43" s="9">
         <v>45665</v>
       </c>
     </row>
     <row r="44" spans="1:73" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A44" s="16"/>
-      <c r="B44" s="16"/>
-      <c r="C44" s="16"/>
-      <c r="D44" s="14"/>
-      <c r="E44" s="14"/>
-      <c r="F44" s="15"/>
+      <c r="A44" s="25"/>
+      <c r="B44" s="25"/>
+      <c r="C44" s="25"/>
+      <c r="D44" s="19"/>
+      <c r="E44" s="19"/>
+      <c r="F44" s="20"/>
       <c r="G44" s="10">
         <v>45820</v>
       </c>
@@ -1780,17 +1788,17 @@
       <c r="BU44" s="7"/>
     </row>
     <row r="45" spans="1:73" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A45" s="16" t="s">
+      <c r="A45" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="B45" s="16"/>
-      <c r="C45" s="16"/>
-      <c r="D45" s="12">
+      <c r="B45" s="25"/>
+      <c r="C45" s="25"/>
+      <c r="D45" s="17">
         <f>SUM(D3:F42)</f>
         <v>84</v>
       </c>
-      <c r="E45" s="12"/>
-      <c r="F45" s="13"/>
+      <c r="E45" s="17"/>
+      <c r="F45" s="18"/>
       <c r="G45" s="9">
         <v>45665</v>
       </c>
@@ -1862,12 +1870,12 @@
       <c r="BU45" s="7"/>
     </row>
     <row r="46" spans="1:73" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A46" s="16"/>
-      <c r="B46" s="16"/>
-      <c r="C46" s="16"/>
-      <c r="D46" s="14"/>
-      <c r="E46" s="14"/>
-      <c r="F46" s="15"/>
+      <c r="A46" s="25"/>
+      <c r="B46" s="25"/>
+      <c r="C46" s="25"/>
+      <c r="D46" s="19"/>
+      <c r="E46" s="19"/>
+      <c r="F46" s="20"/>
       <c r="G46" s="10">
         <v>45820</v>
       </c>
@@ -1940,54 +1948,54 @@
     </row>
   </sheetData>
   <mergeCells count="48">
+    <mergeCell ref="A41:C42"/>
+    <mergeCell ref="D41:F42"/>
+    <mergeCell ref="A43:C44"/>
+    <mergeCell ref="D43:F44"/>
+    <mergeCell ref="A45:C46"/>
+    <mergeCell ref="D45:F46"/>
+    <mergeCell ref="A35:C36"/>
+    <mergeCell ref="D35:F36"/>
+    <mergeCell ref="A37:C38"/>
+    <mergeCell ref="D37:F38"/>
+    <mergeCell ref="A39:C40"/>
+    <mergeCell ref="D39:F40"/>
+    <mergeCell ref="A29:C30"/>
+    <mergeCell ref="D29:F30"/>
+    <mergeCell ref="A31:C32"/>
+    <mergeCell ref="D31:F32"/>
+    <mergeCell ref="A33:C34"/>
+    <mergeCell ref="D33:F34"/>
+    <mergeCell ref="A23:C24"/>
+    <mergeCell ref="D23:F24"/>
+    <mergeCell ref="A25:C26"/>
+    <mergeCell ref="D25:F26"/>
+    <mergeCell ref="A27:C28"/>
+    <mergeCell ref="D27:F28"/>
+    <mergeCell ref="A17:C18"/>
+    <mergeCell ref="D17:F18"/>
+    <mergeCell ref="A19:C20"/>
+    <mergeCell ref="D19:F20"/>
+    <mergeCell ref="A21:C22"/>
+    <mergeCell ref="D21:F22"/>
+    <mergeCell ref="A11:C12"/>
+    <mergeCell ref="D11:F12"/>
+    <mergeCell ref="A13:C14"/>
+    <mergeCell ref="D13:F14"/>
+    <mergeCell ref="A15:C16"/>
+    <mergeCell ref="D15:F16"/>
+    <mergeCell ref="A5:C6"/>
+    <mergeCell ref="D5:F6"/>
+    <mergeCell ref="A7:C8"/>
+    <mergeCell ref="D7:F8"/>
+    <mergeCell ref="A9:C10"/>
+    <mergeCell ref="D9:F10"/>
     <mergeCell ref="BD1:CZ2"/>
     <mergeCell ref="A1:C2"/>
     <mergeCell ref="D1:F2"/>
     <mergeCell ref="G1:BC2"/>
     <mergeCell ref="A3:C4"/>
     <mergeCell ref="D3:F4"/>
-    <mergeCell ref="A5:C6"/>
-    <mergeCell ref="D5:F6"/>
-    <mergeCell ref="A7:C8"/>
-    <mergeCell ref="D7:F8"/>
-    <mergeCell ref="A9:C10"/>
-    <mergeCell ref="D9:F10"/>
-    <mergeCell ref="A11:C12"/>
-    <mergeCell ref="D11:F12"/>
-    <mergeCell ref="A13:C14"/>
-    <mergeCell ref="D13:F14"/>
-    <mergeCell ref="A15:C16"/>
-    <mergeCell ref="D15:F16"/>
-    <mergeCell ref="A17:C18"/>
-    <mergeCell ref="D17:F18"/>
-    <mergeCell ref="A19:C20"/>
-    <mergeCell ref="D19:F20"/>
-    <mergeCell ref="A21:C22"/>
-    <mergeCell ref="D21:F22"/>
-    <mergeCell ref="A23:C24"/>
-    <mergeCell ref="D23:F24"/>
-    <mergeCell ref="A25:C26"/>
-    <mergeCell ref="D25:F26"/>
-    <mergeCell ref="A27:C28"/>
-    <mergeCell ref="D27:F28"/>
-    <mergeCell ref="A29:C30"/>
-    <mergeCell ref="D29:F30"/>
-    <mergeCell ref="A31:C32"/>
-    <mergeCell ref="D31:F32"/>
-    <mergeCell ref="A33:C34"/>
-    <mergeCell ref="D33:F34"/>
-    <mergeCell ref="A35:C36"/>
-    <mergeCell ref="D35:F36"/>
-    <mergeCell ref="A37:C38"/>
-    <mergeCell ref="D37:F38"/>
-    <mergeCell ref="A39:C40"/>
-    <mergeCell ref="D39:F40"/>
-    <mergeCell ref="A41:C42"/>
-    <mergeCell ref="D41:F42"/>
-    <mergeCell ref="A43:C44"/>
-    <mergeCell ref="D43:F44"/>
-    <mergeCell ref="A45:C46"/>
-    <mergeCell ref="D45:F46"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>